<commit_message>
Actualizacion automatica del mapa (2026-03-11 15:32:45)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:R147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Gamarra 1546</t>
+          <t>GAMARRA 1550</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8202,10 +8202,10 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.477231</v>
+        <v>-58.477255</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.58242</v>
+        <v>-34.582395</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -8317,22 +8317,22 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>S01337226</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/6/2026</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>MOLDES 3055</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -8347,12 +8347,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>811627125</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -8367,21 +8367,21 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L93" t="n">
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.494814</v>
+        <v>-58.466692</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.601905</v>
+        <v>-34.555283</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -8391,7 +8391,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8403,7 +8403,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>S01337226</t>
+          <t>S01375612</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MOLDES 3055</t>
+          <t>LACROZE, FEDERICO AV. 2834</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8433,12 +8433,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>811627125</t>
+          <t>811627118</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroidaq</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8460,24 +8460,24 @@
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.466692</v>
+        <v>-58.447177</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.555283</v>
+        <v>-34.574158</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8489,22 +8489,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S01375612</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2/6/2026</t>
+          <t>2/10/2026</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 2834</t>
+          <t>ARENGREEN 1584</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>811627118</t>
+          <t>812440072</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>corroidaq</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -8539,21 +8539,21 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L95" t="n">
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.447177</v>
+        <v>-58.453265</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.574158</v>
+        <v>-34.615073</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8575,7 +8575,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>8322</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -8585,12 +8585,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ARENGREEN 1584</t>
+          <t>ARENAL, CONCEPCION 3814</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -8605,12 +8605,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>812440072</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -8620,36 +8620,36 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L96" t="n">
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.453265</v>
+        <v>-58.447805</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.615073</v>
+        <v>-34.587018</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>ATH-L</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8661,7 +8661,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>8322</t>
+          <t>8323</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ARENAL, CONCEPCION 3814</t>
+          <t>WARNES AV. 2239</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8691,12 +8691,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440018</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -8718,14 +8718,14 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.447805</v>
+        <v>-58.467815</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.587018</v>
+        <v>-34.596225</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>ATH-L</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>8323</t>
+          <t>8324</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>WARNES AV. 2239</t>
+          <t>PAZ SOLDAN 4991</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8777,12 +8777,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>812440018</t>
+          <t>812439995</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base quebrada</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -8797,17 +8797,17 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L98" t="n">
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.467815</v>
+        <v>-58.468466</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.596225</v>
+        <v>-34.594154</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -8833,7 +8833,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>8324</t>
+          <t>8338</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8843,12 +8843,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PAZ SOLDAN 4991</t>
+          <t xml:space="preserve"> GUALEGUAYCHU 4754</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8863,12 +8863,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>812439995</t>
+          <t>812439956</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>base quebrada</t>
+          <t>inclinado, base quebrada</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -8890,10 +8890,10 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.468466</v>
+        <v>-58.518803</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.594154</v>
+        <v>-34.595866</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8919,7 +8919,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>8338</t>
+          <t>8341</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8929,12 +8929,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GUALEGUAYCHU 4754</t>
+          <t>BLANCO ENCALADA 823</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -8949,12 +8949,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>812439956</t>
+          <t>812439941</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>inclinado, base quebrada</t>
+          <t>inclinado base quebrada</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -8976,14 +8976,14 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.518803</v>
+        <v>-58.442692</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.595866</v>
+        <v>-34.549454</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>BLO-B</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9005,22 +9005,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>8341</t>
+          <t>8375</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2/10/2026</t>
+          <t>2/18/2026</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>BLANCO ENCALADA 823</t>
+          <t>DORREGO AV. 2699</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9035,12 +9035,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>812439941</t>
+          <t>812440089</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>inclinado base quebrada</t>
+          <t>base corrodia</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -9055,31 +9055,31 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L101" t="n">
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.442692</v>
+        <v>-58.432807</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.549454</v>
+        <v>-34.574343</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>BLO-B</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9091,22 +9091,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>8375</t>
+          <t>8363</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2/18/2026</t>
+          <t>2/19/2026</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2699</t>
+          <t>BEIRO, FRANCISCO AV. 2435</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -9121,12 +9121,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>812440089</t>
+          <t>812440250</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>base corrodia</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -9148,24 +9148,24 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.432807</v>
+        <v>-58.488914</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.574343</v>
+        <v>-34.59164</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9177,7 +9177,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>8363</t>
+          <t>8367</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9187,7 +9187,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>BEIRO, FRANCISCO AV. 2435</t>
+          <t>CARACAS 3559</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9207,12 +9207,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>812440250</t>
+          <t>812440223</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -9234,10 +9234,10 @@
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.488914</v>
+        <v>-58.487793</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.59164</v>
+        <v>-34.590403</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -9263,7 +9263,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>8367</t>
+          <t>8368</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9273,7 +9273,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CARACAS 3559</t>
+          <t>CARACAS 3519</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -9293,12 +9293,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>812440223</t>
+          <t>812503552</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9320,10 +9320,10 @@
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.487793</v>
+        <v>-58.487627</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.590403</v>
+        <v>-34.590585</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -9349,7 +9349,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>8368</t>
+          <t>8370</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9359,12 +9359,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CARACAS 3519</t>
+          <t>VARELA, JOSE PEDRO 3545</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9379,12 +9379,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>812503552</t>
+          <t>812440219</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -9399,17 +9399,17 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L105" t="n">
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.487627</v>
+        <v>-58.502073</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.590585</v>
+        <v>-34.601294</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9435,7 +9435,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>8370</t>
+          <t>8378</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9445,12 +9445,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>VARELA, JOSE PEDRO 3545</t>
+          <t>ANDONAEGUI 2383</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -9465,12 +9465,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>812440219</t>
+          <t>812440211</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>base corroida inclinada</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -9485,17 +9485,17 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L106" t="n">
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.502073</v>
+        <v>-58.489606</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.601294</v>
+        <v>-34.57655</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -9509,7 +9509,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9521,7 +9521,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>8378</t>
+          <t>8386</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ANDONAEGUI 2383</t>
+          <t>CRAMER 4262</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9551,7 +9551,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>812440211</t>
+          <t>812440206</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9578,14 +9578,14 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.489606</v>
+        <v>-58.476168</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.57655</v>
+        <v>-34.545546</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -9595,7 +9595,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9607,7 +9607,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>8386</t>
+          <t>8387</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9617,7 +9617,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CRAMER 4262</t>
+          <t xml:space="preserve">CRAMER 4322 </t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9637,12 +9637,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>812440206</t>
+          <t>812440204</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>base corroida inclinada</t>
+          <t>base corroida inclnada</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9664,10 +9664,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.476168</v>
+        <v>-58.476454</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.545546</v>
+        <v>-34.544962</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9693,7 +9693,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>8387</t>
+          <t>8382</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9703,12 +9703,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRAMER 4322 </t>
+          <t>SANTO TOME 3588</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9723,12 +9723,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>812440204</t>
+          <t>812440197</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>base corroida inclnada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -9743,21 +9743,21 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L109" t="n">
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.476454</v>
+        <v>-58.4947</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.544962</v>
+        <v>-34.60925</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
@@ -9767,7 +9767,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>DEV-D</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9779,7 +9779,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>8382</t>
+          <t>S00117686</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9789,12 +9789,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SANTO TOME 3588</t>
+          <t>DORREGO AV. 2778</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -9809,12 +9809,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>812440197</t>
+          <t>812440183</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inlinada</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9829,31 +9829,31 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L110" t="n">
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.4947</v>
+        <v>-58.432102</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.60925</v>
+        <v>-34.574248</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>DEV-D</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9865,7 +9865,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>S00117686</t>
+          <t>S00506048</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9875,12 +9875,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2778</t>
+          <t>TERRADA 1088</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -9895,17 +9895,17 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>812440183</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>inlinada</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -9915,31 +9915,31 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L111" t="n">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.432102</v>
+        <v>-58.472866</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.574248</v>
+        <v>-34.620121</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9951,22 +9951,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>S00506048</t>
+          <t>8481</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2/19/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>TERRADA 1088</t>
+          <t>CISNEROS, VIRREY 1610</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9981,17 +9981,17 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440520</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -10008,10 +10008,10 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.472866</v>
+        <v>-58.469727</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.620121</v>
+        <v>-34.612013</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -10025,7 +10025,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>8481</t>
+          <t>8550</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -10047,12 +10047,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>CISNEROS, VIRREY 1610</t>
+          <t>FRAGATA PRES. SARMIENTO 1390</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>812440520</t>
+          <t>812440373</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -10087,17 +10087,17 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L113" t="n">
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.469727</v>
+        <v>-58.456778</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.612013</v>
+        <v>-34.609187</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10123,7 +10123,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>8550</t>
+          <t>S00506118</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10133,12 +10133,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>FRAGATA PRES. SARMIENTO 1390</t>
+          <t>TERRERO 588</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -10153,12 +10153,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>812440373</t>
+          <t>812440289</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -10180,24 +10180,24 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.456778</v>
+        <v>-58.459689</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.609187</v>
+        <v>-34.620032</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>NRA-D</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10209,22 +10209,22 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>S00506118</t>
+          <t>S01295589</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/24/2026</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>TERRERO 588</t>
+          <t>CABILDO AV. 1008</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -10239,7 +10239,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>812440289</t>
+          <t>812440653</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -10266,24 +10266,24 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.459689</v>
+        <v>-58.446714</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.620032</v>
+        <v>-34.569183</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>NRA-D</t>
+          <t>COG-C</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10295,7 +10295,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>S01295589</t>
+          <t>S01406719</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>CABILDO AV. 1008</t>
+          <t>3 DE FEBRERO 4481</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>812440653</t>
+          <t>812440639</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -10345,21 +10345,21 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L116" t="n">
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.446714</v>
+        <v>-58.467166</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.569183</v>
+        <v>-34.539469</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>COG-C</t>
+          <t>BLO-S</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10381,22 +10381,22 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>S01406719</t>
+          <t>S00867165</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2/24/2026</t>
+          <t>2/26/2026</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>3 DE FEBRERO 4481</t>
+          <t xml:space="preserve"> VALLEJOS 2250</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -10411,12 +10411,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>812440639</t>
+          <t>812503628</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -10431,21 +10431,21 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L117" t="n">
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.467166</v>
+        <v>-58.493418</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.539469</v>
+        <v>-34.583307</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>BLO-S</t>
+          <t>PUE-K</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10467,7 +10467,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>S00867165</t>
+          <t>8392</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -10477,12 +10477,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VALLEJOS 2250</t>
+          <t xml:space="preserve">ESTADO PLURINACIONAL DE BOLIVIA 3526 </t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>812503628</t>
+          <t>812503597</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -10524,10 +10524,10 @@
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.493418</v>
+        <v>-58.491306</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.583307</v>
+        <v>-34.592511</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>PUE-K</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10553,7 +10553,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>8392</t>
+          <t>8397</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESTADO PLURINACIONAL DE BOLIVIA 3526 </t>
+          <t>TERRADA 3739</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -10583,12 +10583,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>812503597</t>
+          <t>812503610</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -10610,10 +10610,10 @@
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>-58.491306</v>
+        <v>-58.494807</v>
       </c>
       <c r="N119" t="n">
-        <v>-34.592511</v>
+        <v>-34.592416</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>8397</t>
+          <t>8398</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>TERRADA 3739</t>
+          <t xml:space="preserve"> TERRADA 3695 </t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>812503610</t>
+          <t>812503605</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -10696,10 +10696,10 @@
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>-58.494807</v>
+        <v>-58.494371</v>
       </c>
       <c r="N120" t="n">
-        <v>-34.592416</v>
+        <v>-34.592899</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -10725,22 +10725,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>8398</t>
+          <t>8420</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2/26/2026</t>
+          <t>2/27/2026</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve"> TERRADA 3695 </t>
+          <t>SIMBRON 5855</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -10755,12 +10755,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>812503605</t>
+          <t>812503637</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -10775,21 +10775,21 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L121" t="n">
         <v>1</v>
       </c>
       <c r="M121" t="n">
-        <v>-58.494371</v>
+        <v>-58.527129</v>
       </c>
       <c r="N121" t="n">
-        <v>-34.592899</v>
+        <v>-34.620962</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>DEV-G</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10811,22 +10811,22 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>8420</t>
+          <t>S00208304</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2/27/2026</t>
+          <t>3/2/2026</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SIMBRON 5855</t>
+          <t>CONDE 3080</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -10841,12 +10841,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>812503637</t>
+          <t>812503654</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -10861,21 +10861,21 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L122" t="n">
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-58.527129</v>
+        <v>-58.47322</v>
       </c>
       <c r="N122" t="n">
-        <v>-34.620962</v>
+        <v>-34.558645</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>DEV-G</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -10897,22 +10897,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>S00208304</t>
+          <t>S00106358</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>3/2/2026</t>
+          <t>3/4/2026</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>CONDE 3080</t>
+          <t>TRONADOR 1194</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -10927,7 +10927,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>812503654</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -10954,14 +10954,14 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.47322</v>
+        <v>-58.466138</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.558645</v>
+        <v>-34.579638</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10983,22 +10983,22 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>S00106358</t>
+          <t>S00169078</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>3/4/2026</t>
+          <t>3/5/2026</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TRONADOR 1194</t>
+          <t>LOPEZ, CARLOS ANTONIO 3911</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -11033,21 +11033,21 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L124" t="n">
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.466138</v>
+        <v>-58.516319</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.579638</v>
+        <v>-34.593592</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11069,7 +11069,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>S00169078</t>
+          <t>S00190060</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11079,12 +11079,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LOPEZ, CARLOS ANTONIO 3911</t>
+          <t xml:space="preserve">OBISPO SAN ALBERTO 3176 </t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -11104,7 +11104,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -11119,17 +11119,17 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L125" t="n">
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.516319</v>
+        <v>-58.509545</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.593592</v>
+        <v>-34.584532</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -11143,7 +11143,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>PUE-M</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11155,7 +11155,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>S00190060</t>
+          <t>S00195815</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">OBISPO SAN ALBERTO 3176 </t>
+          <t>PEDRAZA, MANUELA 3345</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -11190,7 +11190,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -11212,14 +11212,14 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>-58.509545</v>
+        <v>-58.474542</v>
       </c>
       <c r="N126" t="n">
-        <v>-34.584532</v>
+        <v>-34.556088</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -11229,7 +11229,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>PUE-M</t>
+          <t>COG-N</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11241,22 +11241,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>S00195815</t>
+          <t>8491</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>3/5/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>PEDRAZA, MANUELA 3345</t>
+          <t>OROÑO, NICASIO 2540</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -11298,14 +11298,14 @@
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>-58.474542</v>
+        <v>-58.459566</v>
       </c>
       <c r="N127" t="n">
-        <v>-34.556088</v>
+        <v>-34.597579</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
@@ -11315,19 +11315,19 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>COG-N</t>
+          <t>NRA-N</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.1NRA</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>8491</t>
+          <t>8496</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -11337,12 +11337,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>OROÑO, NICASIO 2540</t>
+          <t>COSTA RICA 5733</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base corroida inclinada</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -11372,7 +11372,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -11384,36 +11384,36 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>-58.459566</v>
+        <v>-58.436004</v>
       </c>
       <c r="N128" t="n">
-        <v>-34.597579</v>
+        <v>-34.58156</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>NRA-N</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>8496</t>
+          <t>8500</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -11423,12 +11423,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>COSTA RICA 5733</t>
+          <t>LAVOISIER 3556</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -11448,7 +11448,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>base corroida inclinada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -11458,7 +11458,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -11470,24 +11470,24 @@
         <v>1</v>
       </c>
       <c r="M129" t="n">
-        <v>-58.436004</v>
+        <v>-58.502869</v>
       </c>
       <c r="N129" t="n">
-        <v>-34.58156</v>
+        <v>-34.567437</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>PUE-H</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11499,7 +11499,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>8500</t>
+          <t>8508</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11509,12 +11509,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>LAVOISIER 3556</t>
+          <t>NEWBERY, JORGE 3117</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -11534,7 +11534,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -11556,24 +11556,24 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.502869</v>
+        <v>-58.446446</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.567437</v>
+        <v>-34.578293</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>PUE-H</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11585,7 +11585,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>8508</t>
+          <t>8511</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 3117</t>
+          <t>SOLDADO DE LA INDEPENDENCIA 851</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -11642,10 +11642,10 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.446446</v>
+        <v>-58.435443</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.578293</v>
+        <v>-34.56693</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11671,7 +11671,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>8511</t>
+          <t>900009605910</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11681,12 +11681,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SOLDADO DE LA INDEPENDENCIA 851</t>
+          <t xml:space="preserve">BORDABEHERE, ENZO 2801 </t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -11706,7 +11706,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -11721,31 +11721,31 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L132" t="n">
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.435443</v>
+        <v>-58.480297</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.56693</v>
+        <v>-34.600118</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11757,17 +11757,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>900009605910</t>
+          <t>8480</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/5/2026</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">BORDABEHERE, ENZO 2801 </t>
+          <t>NAZCA AV. 3312</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -11807,17 +11807,17 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L133" t="n">
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.480297</v>
+        <v>-58.492236</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.600118</v>
+        <v>-34.598228</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -11831,7 +11831,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11843,22 +11843,22 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>8480</t>
+          <t>8519</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>3/5/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>NAZCA AV. 3312</t>
+          <t>OROÑO, NICASIO 2170</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>Columna Picada</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -11900,10 +11900,10 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.492236</v>
+        <v>-58.460865</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.598228</v>
+        <v>-34.601594</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11917,19 +11917,19 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>NRA-N</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.1NRA</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>8519</t>
+          <t>8528</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11939,12 +11939,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>OROÑO, NICASIO 2170</t>
+          <t>MOLDES 3006</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -11979,21 +11979,21 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L135" t="n">
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.460865</v>
+        <v>-58.466299</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.601594</v>
+        <v>-34.555783</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -12003,19 +12003,19 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>NRA-N</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>8528</t>
+          <t>8534</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12025,12 +12025,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>MOLDES 3006</t>
+          <t xml:space="preserve">ARGERICH 3561 </t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -12065,21 +12065,21 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L136" t="n">
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.466299</v>
+        <v>-58.495986</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.555783</v>
+        <v>-34.595286</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
@@ -12089,7 +12089,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12101,7 +12101,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>8534</t>
+          <t>8435</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARGERICH 3561 </t>
+          <t>DE LOS INCAS AV. 4857</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Columna Picada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -12158,10 +12158,10 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.495986</v>
+        <v>-58.478518</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.595286</v>
+        <v>-34.58436</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12187,7 +12187,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>8435</t>
+          <t>8437</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12197,7 +12197,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>DE LOS INCAS AV. 4857</t>
+          <t>AVALOS 1654</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -12222,7 +12222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -12244,10 +12244,10 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.478518</v>
+        <v>-58.480338</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.58436</v>
+        <v>-34.581544</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12261,7 +12261,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12273,7 +12273,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>8437</t>
+          <t>8438</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>AVALOS 1654</t>
+          <t xml:space="preserve">GAMARRA 1751 </t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12330,10 +12330,10 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.480338</v>
+        <v>-58.479932</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.581544</v>
+        <v>-34.580069</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -12359,7 +12359,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>8438</t>
+          <t>8439</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAMARRA 1751 </t>
+          <t xml:space="preserve">CADIZ 4091 </t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -12394,7 +12394,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12416,10 +12416,10 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.479932</v>
+        <v>-58.478929</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.580069</v>
+        <v>-34.580774</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -12445,7 +12445,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>8439</t>
+          <t>8441</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12455,7 +12455,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">CADIZ 4091 </t>
+          <t xml:space="preserve"> VICTORICA, BENJAMIN, GENERAL, AV. 2330</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12502,10 +12502,10 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.478929</v>
+        <v>-58.478983</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.580774</v>
+        <v>-34.579669</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12531,7 +12531,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>8441</t>
+          <t>8442</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VICTORICA, BENJAMIN, GENERAL, AV. 2330</t>
+          <t>BERNA 2425</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12588,10 +12588,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.478983</v>
+        <v>-58.47814</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.579669</v>
+        <v>-34.581156</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12617,7 +12617,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>8442</t>
+          <t>8443</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>BERNA 2425</t>
+          <t>BERNA 2449</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12674,10 +12674,10 @@
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.47814</v>
+        <v>-58.478248</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.581156</v>
+        <v>-34.581288</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12703,7 +12703,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>8443</t>
+          <t>8447</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>BERNA 2449</t>
+          <t xml:space="preserve">AVALOS 1301 </t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12738,7 +12738,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -12760,10 +12760,10 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.478248</v>
+        <v>-58.477244</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.581288</v>
+        <v>-34.584896</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12777,7 +12777,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12789,7 +12789,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>8447</t>
+          <t>8448</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12799,7 +12799,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">AVALOS 1301 </t>
+          <t>GAMARRA 1504</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12824,7 +12824,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -12846,10 +12846,10 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.477244</v>
+        <v>-58.476783</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.584896</v>
+        <v>-34.582937</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12875,7 +12875,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>8448</t>
+          <t>8450</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>GAMARRA 1504</t>
+          <t>GANDARA 3308</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12910,7 +12910,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -12932,10 +12932,10 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.476783</v>
+        <v>-58.485416</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.582937</v>
+        <v>-34.586085</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12961,7 +12961,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>8450</t>
+          <t>8449</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12971,7 +12971,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>GANDARA 3308</t>
+          <t>GIRIBONE 3355</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -13018,10 +13018,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.485416</v>
+        <v>-58.486528</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.586085</v>
+        <v>-34.585612</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13039,92 +13039,6 @@
         </is>
       </c>
       <c r="R147" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>8449</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>3/9/2026</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>GIRIBONE 3355</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L148" t="n">
-        <v>1</v>
-      </c>
-      <c r="M148" t="n">
-        <v>-58.486528</v>
-      </c>
-      <c r="N148" t="n">
-        <v>-34.585612</v>
-      </c>
-      <c r="O148" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="P148" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q148" t="inlineStr">
-        <is>
-          <t>ATH-S</t>
-        </is>
-      </c>
-      <c r="R148" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-28 12:28:45)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R141"/>
+  <dimension ref="A1:R142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12524,6 +12524,88 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>3/28/2026</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>GIRIBONE 3229</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L142" t="n">
+        <v>1</v>
+      </c>
+      <c r="M142" t="n">
+        <v>-58.485216</v>
+      </c>
+      <c r="N142" t="n">
+        <v>-34.584797</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>ATH-S</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-16 09:13:04)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R188"/>
+  <dimension ref="A1:R192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -16553,6 +16553,334 @@
         </is>
       </c>
       <c r="R188" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr"/>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L189" t="n">
+        <v>1</v>
+      </c>
+      <c r="M189" t="n">
+        <v>-58.444908</v>
+      </c>
+      <c r="N189" t="n">
+        <v>-34.607205</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr"/>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L190" t="n">
+        <v>1</v>
+      </c>
+      <c r="M190" t="n">
+        <v>-58.419576</v>
+      </c>
+      <c r="N190" t="n">
+        <v>-34.621289</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr"/>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L191" t="n">
+        <v>1</v>
+      </c>
+      <c r="M191" t="n">
+        <v>-58.430568</v>
+      </c>
+      <c r="N191" t="n">
+        <v>-34.599485</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>CLI-N</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>M00002</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>4/16/2026</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>MELIAN AV 3893</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>1</v>
+      </c>
+      <c r="M192" t="n">
+        <v>-58.481571</v>
+      </c>
+      <c r="N192" t="n">
+        <v>-34.552784</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-17 09:44:52)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R192"/>
+  <dimension ref="A1:R190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16217,7 +16217,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>00275970</t>
+          <t>00283507</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -16227,12 +16227,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JUJUY AV. 252</t>
+          <t xml:space="preserve">HERRERA 475 </t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -16247,7 +16247,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>812880578</t>
+          <t>812880593</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -16274,14 +16274,14 @@
         <v>1</v>
       </c>
       <c r="M185" t="n">
-        <v>-58.405319</v>
+        <v>-58.378709</v>
       </c>
       <c r="N185" t="n">
-        <v>-34.612931</v>
+        <v>-34.635064</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P185" t="inlineStr">
@@ -16291,7 +16291,7 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>CEN-H</t>
+          <t>CON-H</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -16303,7 +16303,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>00283507</t>
+          <t>00289536</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -16313,12 +16313,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERRERA 475 </t>
+          <t>VALDENEGRO 3554</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -16333,7 +16333,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>812880593</t>
+          <t>812880608</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -16360,24 +16360,24 @@
         <v>1</v>
       </c>
       <c r="M186" t="n">
-        <v>-58.378709</v>
+        <v>-58.490576</v>
       </c>
       <c r="N186" t="n">
-        <v>-34.635064</v>
+        <v>-34.561508</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P186" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>CON-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -16389,22 +16389,22 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>00289536</t>
+          <t>0000001</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/28/2026</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>VALDENEGRO 3554</t>
+          <t>GIRIBONE 3229</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>812880608</t>
+          <t>812880759</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -16446,14 +16446,14 @@
         <v>1</v>
       </c>
       <c r="M187" t="n">
-        <v>-58.490576</v>
+        <v>-58.485216</v>
       </c>
       <c r="N187" t="n">
-        <v>-34.561508</v>
+        <v>-34.584797</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P187" t="inlineStr">
@@ -16463,7 +16463,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -16473,24 +16473,20 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
+      <c r="A188" t="inlineStr"/>
       <c r="B188" t="inlineStr">
         <is>
-          <t>3/28/2026</t>
+          <t>4/14/2026</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>GIRIBONE 3229</t>
+          <t>AV INDEPENDENCIA 3810</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -16505,7 +16501,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>812880759</t>
+          <t>813107750</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -16532,24 +16528,24 @@
         <v>1</v>
       </c>
       <c r="M188" t="n">
-        <v>-58.485216</v>
+        <v>-58.444908</v>
       </c>
       <c r="N188" t="n">
-        <v>-34.584797</v>
+        <v>-34.607205</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -16614,14 +16610,14 @@
         <v>1</v>
       </c>
       <c r="M189" t="n">
-        <v>-58.444908</v>
+        <v>-58.419576</v>
       </c>
       <c r="N189" t="n">
-        <v>-34.607205</v>
+        <v>-34.621289</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P189" t="inlineStr">
@@ -16631,7 +16627,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -16696,14 +16692,14 @@
         <v>1</v>
       </c>
       <c r="M190" t="n">
-        <v>-58.419576</v>
+        <v>-58.430568</v>
       </c>
       <c r="N190" t="n">
-        <v>-34.621289</v>
+        <v>-34.599485</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
@@ -16713,174 +16709,10 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr"/>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>4/14/2026</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>AV INDEPENDENCIA 3810</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>813107750</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L191" t="n">
-        <v>1</v>
-      </c>
-      <c r="M191" t="n">
-        <v>-58.430568</v>
-      </c>
-      <c r="N191" t="n">
-        <v>-34.599485</v>
-      </c>
-      <c r="O191" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P191" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q191" t="inlineStr">
-        <is>
-          <t>CLI-N</t>
-        </is>
-      </c>
-      <c r="R191" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>M00002</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>4/16/2026</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>MELIAN AV 3893</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L192" t="n">
-        <v>1</v>
-      </c>
-      <c r="M192" t="n">
-        <v>-58.481571</v>
-      </c>
-      <c r="N192" t="n">
-        <v>-34.552784</v>
-      </c>
-      <c r="O192" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P192" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q192" t="inlineStr">
-        <is>
-          <t>COG-O</t>
-        </is>
-      </c>
-      <c r="R192" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-20 12:36:43)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R191"/>
+  <dimension ref="A1:R194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16804,6 +16804,252 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr"/>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>1</v>
+      </c>
+      <c r="M192" t="n">
+        <v>-58.437499</v>
+      </c>
+      <c r="N192" t="n">
+        <v>-34.578324</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr"/>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L193" t="n">
+        <v>1</v>
+      </c>
+      <c r="M193" t="n">
+        <v>-58.435547</v>
+      </c>
+      <c r="N193" t="n">
+        <v>-34.576622</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr"/>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>AV INDEPENDENCIA 3810</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>813107750</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L194" t="n">
+        <v>1</v>
+      </c>
+      <c r="M194" t="n">
+        <v>-58.373629</v>
+      </c>
+      <c r="N194" t="n">
+        <v>-34.64417</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>CON-A</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>ARATO-25058.AF.1CON</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-28 08:42:09)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R444"/>
+  <dimension ref="A1:R445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36835,7 +36835,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t xml:space="preserve">10081 </t>
+          <t xml:space="preserve">10080 </t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -36845,7 +36845,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
+          <t>THAMES 549</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -36866,7 +36866,7 @@
       <c r="G430" t="inlineStr"/>
       <c r="H430" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
@@ -36888,10 +36888,10 @@
         <v>1</v>
       </c>
       <c r="M430" t="n">
-        <v>-58.443323</v>
+        <v>-58.442534</v>
       </c>
       <c r="N430" t="n">
-        <v>-34.595549</v>
+        <v>-34.59499</v>
       </c>
       <c r="O430" t="inlineStr">
         <is>
@@ -36917,7 +36917,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t xml:space="preserve">10084 </t>
+          <t xml:space="preserve">10081 </t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -36927,12 +36927,12 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>UGARTE, MANUEL 3258</t>
+          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
@@ -36953,7 +36953,7 @@
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
@@ -36970,24 +36970,24 @@
         <v>1</v>
       </c>
       <c r="M431" t="n">
-        <v>-58.470323</v>
+        <v>-58.443323</v>
       </c>
       <c r="N431" t="n">
-        <v>-34.560769</v>
+        <v>-34.595549</v>
       </c>
       <c r="O431" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P431" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q431" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R431" t="inlineStr">
@@ -36999,7 +36999,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t xml:space="preserve">10087 </t>
+          <t xml:space="preserve">10084 </t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -37009,12 +37009,12 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>CASTILLO 40</t>
+          <t>UGARTE, MANUEL 3258</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
@@ -37052,24 +37052,24 @@
         <v>1</v>
       </c>
       <c r="M432" t="n">
-        <v>-58.430621</v>
+        <v>-58.470323</v>
       </c>
       <c r="N432" t="n">
-        <v>-34.599429</v>
+        <v>-34.560769</v>
       </c>
       <c r="O432" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q432" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R432" t="inlineStr">
@@ -37081,7 +37081,7 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t xml:space="preserve">10102 </t>
+          <t xml:space="preserve">10087 </t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
@@ -37091,7 +37091,7 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>ELCANO AV. 3950</t>
+          <t>CASTILLO 40</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -37112,7 +37112,7 @@
       <c r="G433" t="inlineStr"/>
       <c r="H433" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
@@ -37134,24 +37134,24 @@
         <v>1</v>
       </c>
       <c r="M433" t="n">
-        <v>-58.460457</v>
+        <v>-58.430621</v>
       </c>
       <c r="N433" t="n">
-        <v>-34.582381</v>
+        <v>-34.599429</v>
       </c>
       <c r="O433" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P433" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q433" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R433" t="inlineStr">
@@ -37163,7 +37163,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t xml:space="preserve">10113 </t>
+          <t xml:space="preserve">10102 </t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -37173,12 +37173,12 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>CONCORDIA 4213</t>
+          <t>ELCANO AV. 3950</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -37199,7 +37199,7 @@
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
@@ -37216,14 +37216,14 @@
         <v>1</v>
       </c>
       <c r="M434" t="n">
-        <v>-58.506878</v>
+        <v>-58.460457</v>
       </c>
       <c r="N434" t="n">
-        <v>-34.59474</v>
+        <v>-34.582381</v>
       </c>
       <c r="O434" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P434" t="inlineStr">
@@ -37233,7 +37233,7 @@
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -37245,7 +37245,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t xml:space="preserve">10116 </t>
+          <t xml:space="preserve">10113 </t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -37255,7 +37255,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5858</t>
+          <t>CONCORDIA 4213</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -37276,12 +37276,12 @@
       <c r="G435" t="inlineStr"/>
       <c r="H435" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
@@ -37298,10 +37298,10 @@
         <v>1</v>
       </c>
       <c r="M435" t="n">
-        <v>-58.496239</v>
+        <v>-58.506878</v>
       </c>
       <c r="N435" t="n">
-        <v>-34.564136</v>
+        <v>-34.59474</v>
       </c>
       <c r="O435" t="inlineStr">
         <is>
@@ -37315,7 +37315,7 @@
       </c>
       <c r="Q435" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R435" t="inlineStr">
@@ -37327,7 +37327,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t xml:space="preserve">10119 </t>
+          <t xml:space="preserve">10116 </t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -37337,7 +37337,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5900</t>
+          <t>TRIUNVIRATO AV. 5858</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
@@ -37358,12 +37358,12 @@
       <c r="G436" t="inlineStr"/>
       <c r="H436" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
@@ -37373,17 +37373,17 @@
       </c>
       <c r="K436" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L436" t="n">
         <v>1</v>
       </c>
       <c r="M436" t="n">
-        <v>-58.496593</v>
+        <v>-58.496239</v>
       </c>
       <c r="N436" t="n">
-        <v>-34.563646</v>
+        <v>-34.564136</v>
       </c>
       <c r="O436" t="inlineStr">
         <is>
@@ -37409,7 +37409,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t xml:space="preserve">10126 </t>
+          <t xml:space="preserve">10119 </t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -37419,7 +37419,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
+          <t>TRIUNVIRATO AV. 5900</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -37440,12 +37440,12 @@
       <c r="G437" t="inlineStr"/>
       <c r="H437" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
@@ -37455,21 +37455,21 @@
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L437" t="n">
         <v>1</v>
       </c>
       <c r="M437" t="n">
-        <v>-58.482122</v>
+        <v>-58.496593</v>
       </c>
       <c r="N437" t="n">
-        <v>-34.570386</v>
+        <v>-34.563646</v>
       </c>
       <c r="O437" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P437" t="inlineStr">
@@ -37479,7 +37479,7 @@
       </c>
       <c r="Q437" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R437" t="inlineStr">
@@ -37491,7 +37491,7 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t xml:space="preserve">10133 </t>
+          <t xml:space="preserve">10126 </t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -37501,7 +37501,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
+          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
@@ -37522,12 +37522,12 @@
       <c r="G438" t="inlineStr"/>
       <c r="H438" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
@@ -37544,14 +37544,14 @@
         <v>1</v>
       </c>
       <c r="M438" t="n">
-        <v>-58.453426</v>
+        <v>-58.482122</v>
       </c>
       <c r="N438" t="n">
-        <v>-34.600121</v>
+        <v>-34.570386</v>
       </c>
       <c r="O438" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P438" t="inlineStr">
@@ -37561,7 +37561,7 @@
       </c>
       <c r="Q438" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R438" t="inlineStr">
@@ -37573,7 +37573,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t xml:space="preserve">10136 </t>
+          <t xml:space="preserve">10133 </t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -37583,12 +37583,12 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 2118</t>
+          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
@@ -37626,10 +37626,10 @@
         <v>1</v>
       </c>
       <c r="M439" t="n">
-        <v>-58.456381</v>
+        <v>-58.453426</v>
       </c>
       <c r="N439" t="n">
-        <v>-34.60076</v>
+        <v>-34.600121</v>
       </c>
       <c r="O439" t="inlineStr">
         <is>
@@ -37643,7 +37643,7 @@
       </c>
       <c r="Q439" t="inlineStr">
         <is>
-          <t>NRA-G</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R439" t="inlineStr">
@@ -37655,7 +37655,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t xml:space="preserve">10145 </t>
+          <t xml:space="preserve">10136 </t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -37665,12 +37665,12 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>DONADO 2554</t>
+          <t>REPETTO, NICOLAS, DR. 2118</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
@@ -37708,14 +37708,14 @@
         <v>1</v>
       </c>
       <c r="M440" t="n">
-        <v>-58.478634</v>
+        <v>-58.456381</v>
       </c>
       <c r="N440" t="n">
-        <v>-34.569063</v>
+        <v>-34.60076</v>
       </c>
       <c r="O440" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P440" t="inlineStr">
@@ -37725,7 +37725,7 @@
       </c>
       <c r="Q440" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>NRA-G</t>
         </is>
       </c>
       <c r="R440" t="inlineStr">
@@ -37737,7 +37737,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t xml:space="preserve">10147 </t>
+          <t xml:space="preserve">10145 </t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -37747,7 +37747,7 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>ROOSEVELT FRANKLIN D. 4336</t>
+          <t>DONADO 2554</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
@@ -37768,12 +37768,12 @@
       <c r="G441" t="inlineStr"/>
       <c r="H441" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J441" t="inlineStr">
@@ -37783,17 +37783,17 @@
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L441" t="n">
         <v>1</v>
       </c>
       <c r="M441" t="n">
-        <v>-58.479316</v>
+        <v>-58.478634</v>
       </c>
       <c r="N441" t="n">
-        <v>-34.568762</v>
+        <v>-34.569063</v>
       </c>
       <c r="O441" t="inlineStr">
         <is>
@@ -37819,7 +37819,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t xml:space="preserve">10148 </t>
+          <t xml:space="preserve">10147 </t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -37829,7 +37829,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>ACHA, MARIANO, GRAL. 2595</t>
+          <t>ROOSEVELT FRANKLIN D. 4336</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
@@ -37850,12 +37850,12 @@
       <c r="G442" t="inlineStr"/>
       <c r="H442" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J442" t="inlineStr">
@@ -37865,17 +37865,17 @@
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L442" t="n">
         <v>1</v>
       </c>
       <c r="M442" t="n">
-        <v>-58.479759</v>
+        <v>-58.479316</v>
       </c>
       <c r="N442" t="n">
-        <v>-34.569184</v>
+        <v>-34.568762</v>
       </c>
       <c r="O442" t="inlineStr">
         <is>
@@ -37901,7 +37901,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>10113B</t>
+          <t xml:space="preserve">10148 </t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -37911,7 +37911,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>CONCORDIA 4213</t>
+          <t>ACHA, MARIANO, GRAL. 2595</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
@@ -37932,12 +37932,12 @@
       <c r="G443" t="inlineStr"/>
       <c r="H443" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J443" t="inlineStr">
@@ -37954,14 +37954,14 @@
         <v>1</v>
       </c>
       <c r="M443" t="n">
-        <v>-58.506878</v>
+        <v>-58.479759</v>
       </c>
       <c r="N443" t="n">
-        <v>-34.59474</v>
+        <v>-34.569184</v>
       </c>
       <c r="O443" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P443" t="inlineStr">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="Q443" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R443" t="inlineStr">
@@ -37983,7 +37983,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>10116B</t>
+          <t>10113B</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
@@ -37993,7 +37993,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5858</t>
+          <t>CONCORDIA 4213</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
@@ -38036,27 +38036,109 @@
         <v>1</v>
       </c>
       <c r="M444" t="n">
+        <v>-58.506878</v>
+      </c>
+      <c r="N444" t="n">
+        <v>-34.59474</v>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P444" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q444" t="inlineStr">
+        <is>
+          <t>PUE-O</t>
+        </is>
+      </c>
+      <c r="R444" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>10116B</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>TRIUNVIRATO AV. 5858</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr"/>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>COLUMNA INCLINADA</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L445" t="n">
+        <v>1</v>
+      </c>
+      <c r="M445" t="n">
         <v>-58.496239</v>
       </c>
-      <c r="N444" t="n">
+      <c r="N445" t="n">
         <v>-34.564136</v>
       </c>
-      <c r="O444" t="inlineStr">
+      <c r="O445" t="inlineStr">
         <is>
           <t>Paternal</t>
         </is>
       </c>
-      <c r="P444" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q444" t="inlineStr">
+      <c r="P445" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q445" t="inlineStr">
         <is>
           <t>PUE-F</t>
         </is>
       </c>
-      <c r="R444" t="inlineStr">
+      <c r="R445" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:05:50)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -29007,7 +29007,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G334" t="inlineStr"/>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>814109727</t>
+        </is>
+      </c>
       <c r="H334" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -29171,7 +29175,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G336" t="inlineStr"/>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>814109768</t>
+        </is>
+      </c>
       <c r="H336" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -31057,7 +31065,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G359" t="inlineStr"/>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>814109792</t>
+        </is>
+      </c>
       <c r="H359" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -31221,7 +31233,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G361" t="inlineStr"/>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>814109807</t>
+        </is>
+      </c>
       <c r="H361" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -32287,7 +32303,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G374" t="inlineStr"/>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>814109811</t>
+        </is>
+      </c>
       <c r="H374" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -32369,7 +32389,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G375" t="inlineStr"/>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>814109827</t>
+        </is>
+      </c>
       <c r="H375" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -32451,7 +32475,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G376" t="inlineStr"/>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>814109832</t>
+        </is>
+      </c>
       <c r="H376" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -34279,7 +34307,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G398" t="inlineStr"/>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>814109844</t>
+        </is>
+      </c>
       <c r="H398" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-08 12:33:56)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R373"/>
+  <dimension ref="A1:R371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27537,7 +27537,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t xml:space="preserve">9957 </t>
+          <t xml:space="preserve">9960 </t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -27547,7 +27547,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>JURAMENTO 5347</t>
+          <t>BUCARELLI 1995</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -27560,11 +27560,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr">
-        <is>
-          <t>814111217</t>
-        </is>
-      </c>
+      <c r="F317" t="inlineStr"/>
       <c r="G317" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -27572,7 +27568,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -27582,7 +27578,7 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -27594,10 +27590,10 @@
         <v>1</v>
       </c>
       <c r="M317" t="n">
-        <v>-58.485468</v>
+        <v>-58.484744</v>
       </c>
       <c r="N317" t="n">
-        <v>-34.579765</v>
+        <v>-34.579576</v>
       </c>
       <c r="O317" t="inlineStr">
         <is>
@@ -27623,7 +27619,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t xml:space="preserve">9960 </t>
+          <t xml:space="preserve">9963 </t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -27633,7 +27629,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>BUCARELLI 1995</t>
+          <t xml:space="preserve">BARZANA 1814 </t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -27646,7 +27642,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F318" t="inlineStr"/>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>814111225</t>
+        </is>
+      </c>
       <c r="G318" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -27654,7 +27654,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -27676,10 +27676,10 @@
         <v>1</v>
       </c>
       <c r="M318" t="n">
-        <v>-58.484744</v>
+        <v>-58.485279</v>
       </c>
       <c r="N318" t="n">
-        <v>-34.579576</v>
+        <v>-34.582509</v>
       </c>
       <c r="O318" t="inlineStr">
         <is>
@@ -27693,7 +27693,7 @@
       </c>
       <c r="Q318" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R318" t="inlineStr">
@@ -27705,7 +27705,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t xml:space="preserve">9961 </t>
+          <t xml:space="preserve">9964 </t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -27715,12 +27715,12 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>JURAMENTO 5261</t>
+          <t>BARZANA 1844</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -27730,7 +27730,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>814111218</t>
+          <t>814111227</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
@@ -27762,10 +27762,10 @@
         <v>1</v>
       </c>
       <c r="M319" t="n">
-        <v>-58.484396</v>
+        <v>-58.485434</v>
       </c>
       <c r="N319" t="n">
-        <v>-34.579179</v>
+        <v>-34.582311</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -27779,7 +27779,7 @@
       </c>
       <c r="Q319" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R319" t="inlineStr">
@@ -27791,7 +27791,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t xml:space="preserve">9963 </t>
+          <t xml:space="preserve">9965 </t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -27801,7 +27801,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t xml:space="preserve">BARZANA 1814 </t>
+          <t>ALTOLAGUIRRE 1813</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -27816,7 +27816,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>814111225</t>
+          <t>814111230</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -27848,10 +27848,10 @@
         <v>1</v>
       </c>
       <c r="M320" t="n">
-        <v>-58.485279</v>
+        <v>-58.486073</v>
       </c>
       <c r="N320" t="n">
-        <v>-34.582509</v>
+        <v>-34.582965</v>
       </c>
       <c r="O320" t="inlineStr">
         <is>
@@ -27877,7 +27877,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t xml:space="preserve">9964 </t>
+          <t xml:space="preserve">9966 </t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -27887,7 +27887,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>BARZANA 1844</t>
+          <t>BURELA 1845</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -27902,7 +27902,7 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>814111227</t>
+          <t>814109792</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -27912,7 +27912,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -27934,10 +27934,10 @@
         <v>1</v>
       </c>
       <c r="M321" t="n">
-        <v>-58.485434</v>
+        <v>-58.487319</v>
       </c>
       <c r="N321" t="n">
-        <v>-34.582311</v>
+        <v>-34.583364</v>
       </c>
       <c r="O321" t="inlineStr">
         <is>
@@ -27951,7 +27951,7 @@
       </c>
       <c r="Q321" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>PUE-K</t>
         </is>
       </c>
       <c r="R321" t="inlineStr">
@@ -27963,7 +27963,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t xml:space="preserve">9965 </t>
+          <t xml:space="preserve">9967 </t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -27973,7 +27973,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>ALTOLAGUIRRE 1813</t>
+          <t>CERETTI 1850</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -27988,7 +27988,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>814111230</t>
+          <t>814111327</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -28020,10 +28020,10 @@
         <v>1</v>
       </c>
       <c r="M322" t="n">
-        <v>-58.486073</v>
+        <v>-58.488493</v>
       </c>
       <c r="N322" t="n">
-        <v>-34.582965</v>
+        <v>-34.583983</v>
       </c>
       <c r="O322" t="inlineStr">
         <is>
@@ -28037,7 +28037,7 @@
       </c>
       <c r="Q322" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>PUE-K</t>
         </is>
       </c>
       <c r="R322" t="inlineStr">
@@ -28049,7 +28049,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t xml:space="preserve">9966 </t>
+          <t xml:space="preserve">9969 </t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -28059,12 +28059,12 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>BURELA 1845</t>
+          <t>MONTAÑESES 1910</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -28074,7 +28074,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>814109792</t>
+          <t>814109807</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -28106,14 +28106,14 @@
         <v>1</v>
       </c>
       <c r="M323" t="n">
-        <v>-58.487319</v>
+        <v>-58.447489</v>
       </c>
       <c r="N323" t="n">
-        <v>-34.583364</v>
+        <v>-34.559091</v>
       </c>
       <c r="O323" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P323" t="inlineStr">
@@ -28123,7 +28123,7 @@
       </c>
       <c r="Q323" t="inlineStr">
         <is>
-          <t>PUE-K</t>
+          <t>BLO-A</t>
         </is>
       </c>
       <c r="R323" t="inlineStr">
@@ -28135,7 +28135,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t xml:space="preserve">9967 </t>
+          <t xml:space="preserve">9970 </t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -28145,7 +28145,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>CERETTI 1850</t>
+          <t>ECHEVERRIA 5051</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -28160,7 +28160,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>814111327</t>
+          <t>814111395</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -28192,10 +28192,10 @@
         <v>1</v>
       </c>
       <c r="M324" t="n">
-        <v>-58.488493</v>
+        <v>-58.481099</v>
       </c>
       <c r="N324" t="n">
-        <v>-34.583983</v>
+        <v>-34.578912</v>
       </c>
       <c r="O324" t="inlineStr">
         <is>
@@ -28209,7 +28209,7 @@
       </c>
       <c r="Q324" t="inlineStr">
         <is>
-          <t>PUE-K</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R324" t="inlineStr">
@@ -28221,7 +28221,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t xml:space="preserve">9969 </t>
+          <t xml:space="preserve">9971 </t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -28231,12 +28231,12 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>MONTAÑESES 1910</t>
+          <t>ECHEVERRIA 5021</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -28246,7 +28246,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>814109807</t>
+          <t>814111401</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
@@ -28256,7 +28256,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
@@ -28278,14 +28278,14 @@
         <v>1</v>
       </c>
       <c r="M325" t="n">
-        <v>-58.447489</v>
+        <v>-58.480634</v>
       </c>
       <c r="N325" t="n">
-        <v>-34.559091</v>
+        <v>-34.578647</v>
       </c>
       <c r="O325" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P325" t="inlineStr">
@@ -28295,7 +28295,7 @@
       </c>
       <c r="Q325" t="inlineStr">
         <is>
-          <t>BLO-A</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R325" t="inlineStr">
@@ -28307,7 +28307,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t xml:space="preserve">9970 </t>
+          <t xml:space="preserve">9993 </t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>ECHEVERRIA 5051</t>
+          <t>MONROE 5212</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>814111395</t>
+          <t>814111591</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
@@ -28364,10 +28364,10 @@
         <v>1</v>
       </c>
       <c r="M326" t="n">
-        <v>-58.481099</v>
+        <v>-58.487529</v>
       </c>
       <c r="N326" t="n">
-        <v>-34.578912</v>
+        <v>-34.575028</v>
       </c>
       <c r="O326" t="inlineStr">
         <is>
@@ -28381,7 +28381,7 @@
       </c>
       <c r="Q326" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R326" t="inlineStr">
@@ -28393,7 +28393,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t xml:space="preserve">9971 </t>
+          <t xml:space="preserve">9996 </t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -28403,7 +28403,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>ECHEVERRIA 5021</t>
+          <t>ZAMUDIO 4784</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -28418,7 +28418,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>814111401</t>
+          <t>814111621</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -28450,10 +28450,10 @@
         <v>1</v>
       </c>
       <c r="M327" t="n">
-        <v>-58.480634</v>
+        <v>-58.497199</v>
       </c>
       <c r="N327" t="n">
-        <v>-34.578647</v>
+        <v>-34.582097</v>
       </c>
       <c r="O327" t="inlineStr">
         <is>
@@ -28467,7 +28467,7 @@
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>PUE-M</t>
         </is>
       </c>
       <c r="R327" t="inlineStr">
@@ -28479,22 +28479,22 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t xml:space="preserve">9993 </t>
+          <t xml:space="preserve">8804 </t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>MONROE 5212</t>
+          <t>LOPEZ MERINO, FRANCISCO 3988</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -28504,7 +28504,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>814111591</t>
+          <t>814108011</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -28514,7 +28514,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -28536,10 +28536,10 @@
         <v>1</v>
       </c>
       <c r="M328" t="n">
-        <v>-58.487529</v>
+        <v>-58.493486</v>
       </c>
       <c r="N328" t="n">
-        <v>-34.575028</v>
+        <v>-34.589105</v>
       </c>
       <c r="O328" t="inlineStr">
         <is>
@@ -28553,7 +28553,7 @@
       </c>
       <c r="Q328" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R328" t="inlineStr">
@@ -28565,17 +28565,17 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t xml:space="preserve">9996 </t>
+          <t xml:space="preserve">8962 </t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ZAMUDIO 4784</t>
+          <t>CONGRESO AV. 5856</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -28590,7 +28590,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>814111621</t>
+          <t>814108043</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -28600,7 +28600,7 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
@@ -28622,10 +28622,10 @@
         <v>1</v>
       </c>
       <c r="M329" t="n">
-        <v>-58.497199</v>
+        <v>-58.499051</v>
       </c>
       <c r="N329" t="n">
-        <v>-34.582097</v>
+        <v>-34.57451</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -28639,7 +28639,7 @@
       </c>
       <c r="Q329" t="inlineStr">
         <is>
-          <t>PUE-M</t>
+          <t>PUE-I</t>
         </is>
       </c>
       <c r="R329" t="inlineStr">
@@ -28651,7 +28651,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t xml:space="preserve">8804 </t>
+          <t xml:space="preserve">8982 </t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -28661,12 +28661,12 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>LOPEZ MERINO, FRANCISCO 3988</t>
+          <t>LOPEZ, CARLOS ANTONIO 2197</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -28676,7 +28676,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>814108011</t>
+          <t>814108057</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -28708,10 +28708,10 @@
         <v>1</v>
       </c>
       <c r="M330" t="n">
-        <v>-58.493486</v>
+        <v>-58.494928</v>
       </c>
       <c r="N330" t="n">
-        <v>-34.589105</v>
+        <v>-34.580378</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -28725,7 +28725,7 @@
       </c>
       <c r="Q330" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>PUE-M</t>
         </is>
       </c>
       <c r="R330" t="inlineStr">
@@ -28737,7 +28737,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t xml:space="preserve">8962 </t>
+          <t xml:space="preserve">10024 </t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -28747,7 +28747,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>CONGRESO AV. 5856</t>
+          <t>IBERA 6146</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -28762,7 +28762,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>814108043</t>
+          <t>814111657</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -28772,7 +28772,7 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
@@ -28794,10 +28794,10 @@
         <v>1</v>
       </c>
       <c r="M331" t="n">
-        <v>-58.499051</v>
+        <v>-58.502338</v>
       </c>
       <c r="N331" t="n">
-        <v>-34.57451</v>
+        <v>-34.573275</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -28823,7 +28823,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t xml:space="preserve">8982 </t>
+          <t xml:space="preserve">10025 </t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -28833,12 +28833,12 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>LOPEZ, CARLOS ANTONIO 2197</t>
+          <t>JUSTO, JUAN B. AV. 3073</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -28848,7 +28848,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>814108057</t>
+          <t>814111671</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
@@ -28858,7 +28858,7 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -28880,10 +28880,10 @@
         <v>1</v>
       </c>
       <c r="M332" t="n">
-        <v>-58.494928</v>
+        <v>-58.449604</v>
       </c>
       <c r="N332" t="n">
-        <v>-34.580378</v>
+        <v>-34.598286</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -28897,7 +28897,7 @@
       </c>
       <c r="Q332" t="inlineStr">
         <is>
-          <t>PUE-M</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R332" t="inlineStr">
@@ -28909,7 +28909,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t xml:space="preserve">10024 </t>
+          <t xml:space="preserve">10026 </t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -28919,7 +28919,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>IBERA 6146</t>
+          <t>HUMBOLDT 47</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -28934,7 +28934,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>814111657</t>
+          <t>814111684</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -28966,10 +28966,10 @@
         <v>1</v>
       </c>
       <c r="M333" t="n">
-        <v>-58.502338</v>
+        <v>-58.451981</v>
       </c>
       <c r="N333" t="n">
-        <v>-34.573275</v>
+        <v>-34.597952</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="Q333" t="inlineStr">
         <is>
-          <t>PUE-I</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R333" t="inlineStr">
@@ -28995,22 +28995,22 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t xml:space="preserve">10025 </t>
+          <t xml:space="preserve">10027 </t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/7/2026</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>JUSTO, JUAN B. AV. 3073</t>
+          <t>HUMBOLDT 37</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -29020,7 +29020,7 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>814111671</t>
+          <t>814111686</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
@@ -29052,10 +29052,10 @@
         <v>1</v>
       </c>
       <c r="M334" t="n">
-        <v>-58.449604</v>
+        <v>-58.452157</v>
       </c>
       <c r="N334" t="n">
-        <v>-34.598286</v>
+        <v>-34.598081</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t xml:space="preserve">10026 </t>
+          <t xml:space="preserve">10028 </t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -29091,12 +29091,12 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>HUMBOLDT 47</t>
+          <t>HUMBOLDT 23</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -29104,11 +29104,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr">
-        <is>
-          <t>814111684</t>
-        </is>
-      </c>
+      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -29121,12 +29117,12 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
@@ -29138,10 +29134,10 @@
         <v>1</v>
       </c>
       <c r="M335" t="n">
-        <v>-58.451981</v>
+        <v>-58.452473</v>
       </c>
       <c r="N335" t="n">
-        <v>-34.597952</v>
+        <v>-34.598316</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -29167,22 +29163,22 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t xml:space="preserve">10027 </t>
+          <t xml:space="preserve">10030 </t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>5/7/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>HUMBOLDT 37</t>
+          <t>SUSINI, ANTONIO, CNEL. 2190</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -29192,7 +29188,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>814111686</t>
+          <t>814111692</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -29224,10 +29220,10 @@
         <v>1</v>
       </c>
       <c r="M336" t="n">
-        <v>-58.452157</v>
+        <v>-58.452997</v>
       </c>
       <c r="N336" t="n">
-        <v>-34.598081</v>
+        <v>-34.597674</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -29253,7 +29249,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t xml:space="preserve">10028 </t>
+          <t xml:space="preserve">9053 </t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -29263,7 +29259,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>HUMBOLDT 23</t>
+          <t>FRAGA 1848</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -29276,7 +29272,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>814108072</t>
+        </is>
+      </c>
       <c r="G337" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -29284,17 +29284,17 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
@@ -29306,14 +29306,14 @@
         <v>1</v>
       </c>
       <c r="M337" t="n">
-        <v>-58.452473</v>
+        <v>-58.468977</v>
       </c>
       <c r="N337" t="n">
-        <v>-34.598316</v>
+        <v>-34.582742</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P337" t="inlineStr">
@@ -29323,7 +29323,7 @@
       </c>
       <c r="Q337" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">
@@ -29335,7 +29335,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t xml:space="preserve">10030 </t>
+          <t>S00527817</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -29345,7 +29345,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>SUSINI, ANTONIO, CNEL. 2190</t>
+          <t>TINOGASTA 2561</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -29358,11 +29358,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr">
-        <is>
-          <t>814111692</t>
-        </is>
-      </c>
+      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -29370,12 +29366,12 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J338" t="inlineStr">
@@ -29392,10 +29388,10 @@
         <v>1</v>
       </c>
       <c r="M338" t="n">
-        <v>-58.452997</v>
+        <v>-58.487709</v>
       </c>
       <c r="N338" t="n">
-        <v>-34.597674</v>
+        <v>-34.595778</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -29409,7 +29405,7 @@
       </c>
       <c r="Q338" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R338" t="inlineStr">
@@ -29421,7 +29417,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t xml:space="preserve">9053 </t>
+          <t xml:space="preserve">10049 </t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -29431,7 +29427,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>FRAGA 1848</t>
+          <t>HEREDIA 1295</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
@@ -29446,7 +29442,7 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>814108072</t>
+          <t>814111714</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -29456,7 +29452,7 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -29478,10 +29474,10 @@
         <v>1</v>
       </c>
       <c r="M339" t="n">
-        <v>-58.468977</v>
+        <v>-58.463173</v>
       </c>
       <c r="N339" t="n">
-        <v>-34.582742</v>
+        <v>-34.57859</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -29495,7 +29491,7 @@
       </c>
       <c r="Q339" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R339" t="inlineStr">
@@ -29507,22 +29503,22 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>S00527817</t>
+          <t xml:space="preserve">10057 </t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/7/2026</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>TINOGASTA 2561</t>
+          <t>TERRADA 4593</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -29530,7 +29526,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr"/>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>814109844</t>
+        </is>
+      </c>
       <c r="G340" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -29538,12 +29538,12 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J340" t="inlineStr">
@@ -29560,10 +29560,10 @@
         <v>1</v>
       </c>
       <c r="M340" t="n">
-        <v>-58.487709</v>
+        <v>-58.500145</v>
       </c>
       <c r="N340" t="n">
-        <v>-34.595778</v>
+        <v>-34.586507</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -29577,7 +29577,7 @@
       </c>
       <c r="Q340" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>PUE-K</t>
         </is>
       </c>
       <c r="R340" t="inlineStr">
@@ -29589,7 +29589,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t xml:space="preserve">10049 </t>
+          <t xml:space="preserve">10060 </t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -29599,12 +29599,12 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>HEREDIA 1295</t>
+          <t xml:space="preserve">AREVALO 2951 </t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -29614,7 +29614,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>814111714</t>
+          <t>814108282</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -29624,7 +29624,7 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
@@ -29646,24 +29646,24 @@
         <v>1</v>
       </c>
       <c r="M341" t="n">
-        <v>-58.463173</v>
+        <v>-58.430757</v>
       </c>
       <c r="N341" t="n">
-        <v>-34.57859</v>
+        <v>-34.571657</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P341" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q341" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R341" t="inlineStr">
@@ -29675,22 +29675,22 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t xml:space="preserve">10057 </t>
+          <t xml:space="preserve">10069 </t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>5/7/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>TERRADA 4593</t>
+          <t xml:space="preserve">CORDOBA AV. 5387 </t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>814109844</t>
+          <t>814111735</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -29710,7 +29710,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -29732,24 +29732,24 @@
         <v>1</v>
       </c>
       <c r="M342" t="n">
-        <v>-58.500145</v>
+        <v>-58.437815</v>
       </c>
       <c r="N342" t="n">
-        <v>-34.586507</v>
+        <v>-34.589036</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P342" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q342" t="inlineStr">
         <is>
-          <t>PUE-K</t>
+          <t>VCR-I</t>
         </is>
       </c>
       <c r="R342" t="inlineStr">
@@ -29761,7 +29761,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">10060 </t>
+          <t xml:space="preserve">10070 </t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -29771,7 +29771,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t xml:space="preserve">AREVALO 2951 </t>
+          <t>NUÑEZ 4634</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
@@ -29786,7 +29786,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>814108282</t>
+          <t>814108373</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -29796,7 +29796,7 @@
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
@@ -29818,24 +29818,24 @@
         <v>1</v>
       </c>
       <c r="M343" t="n">
-        <v>-58.430757</v>
+        <v>-58.487462</v>
       </c>
       <c r="N343" t="n">
-        <v>-34.571657</v>
+        <v>-34.561007</v>
       </c>
       <c r="O343" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P343" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q343" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R343" t="inlineStr">
@@ -29847,7 +29847,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t xml:space="preserve">10069 </t>
+          <t xml:space="preserve">10079 </t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -29857,7 +29857,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t xml:space="preserve">CORDOBA AV. 5387 </t>
+          <t>VILLARROEL 1035</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -29872,7 +29872,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>814111735</t>
+          <t>814111768</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -29904,10 +29904,10 @@
         <v>1</v>
       </c>
       <c r="M344" t="n">
-        <v>-58.437815</v>
+        <v>-58.442939</v>
       </c>
       <c r="N344" t="n">
-        <v>-34.589036</v>
+        <v>-34.594741</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -29921,7 +29921,7 @@
       </c>
       <c r="Q344" t="inlineStr">
         <is>
-          <t>VCR-I</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R344" t="inlineStr">
@@ -29933,7 +29933,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t xml:space="preserve">10070 </t>
+          <t xml:space="preserve">10080 </t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -29943,12 +29943,12 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>NUÑEZ 4634</t>
+          <t>THAMES 549</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -29958,7 +29958,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>814108373</t>
+          <t>814111773</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -29968,7 +29968,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -29990,24 +29990,24 @@
         <v>1</v>
       </c>
       <c r="M345" t="n">
-        <v>-58.487462</v>
+        <v>-58.442534</v>
       </c>
       <c r="N345" t="n">
-        <v>-34.561007</v>
+        <v>-34.59499</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P345" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q345" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R345" t="inlineStr">
@@ -30019,7 +30019,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t xml:space="preserve">10079 </t>
+          <t xml:space="preserve">10081 </t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -30029,7 +30029,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>VILLARROEL 1035</t>
+          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -30044,7 +30044,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>814111768</t>
+          <t>814111776</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -30054,7 +30054,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -30076,10 +30076,10 @@
         <v>1</v>
       </c>
       <c r="M346" t="n">
-        <v>-58.442939</v>
+        <v>-58.443323</v>
       </c>
       <c r="N346" t="n">
-        <v>-34.594741</v>
+        <v>-34.595549</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -30105,7 +30105,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t xml:space="preserve">10080 </t>
+          <t xml:space="preserve">10084 </t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -30115,12 +30115,12 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>THAMES 549</t>
+          <t>UGARTE, MANUEL 3258</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -30130,7 +30130,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>814111773</t>
+          <t>814108396</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -30140,7 +30140,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -30162,24 +30162,24 @@
         <v>1</v>
       </c>
       <c r="M347" t="n">
-        <v>-58.442534</v>
+        <v>-58.470323</v>
       </c>
       <c r="N347" t="n">
-        <v>-34.59499</v>
+        <v>-34.560769</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P347" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q347" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R347" t="inlineStr">
@@ -30191,7 +30191,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t xml:space="preserve">10081 </t>
+          <t xml:space="preserve">10087 </t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -30201,7 +30201,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
+          <t>CASTILLO 40</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -30216,7 +30216,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>814111776</t>
+          <t>814108420</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -30248,10 +30248,10 @@
         <v>1</v>
       </c>
       <c r="M348" t="n">
-        <v>-58.443323</v>
+        <v>-58.430621</v>
       </c>
       <c r="N348" t="n">
-        <v>-34.595549</v>
+        <v>-34.599429</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -30265,7 +30265,7 @@
       </c>
       <c r="Q348" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R348" t="inlineStr">
@@ -30277,7 +30277,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t xml:space="preserve">10084 </t>
+          <t xml:space="preserve">10102 </t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -30287,12 +30287,12 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>UGARTE, MANUEL 3258</t>
+          <t>ELCANO AV. 3950</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -30302,7 +30302,7 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>814108396</t>
+          <t>814108464</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -30312,7 +30312,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
@@ -30334,10 +30334,10 @@
         <v>1</v>
       </c>
       <c r="M349" t="n">
-        <v>-58.470323</v>
+        <v>-58.460457</v>
       </c>
       <c r="N349" t="n">
-        <v>-34.560769</v>
+        <v>-34.582381</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -30351,7 +30351,7 @@
       </c>
       <c r="Q349" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R349" t="inlineStr">
@@ -30363,7 +30363,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t xml:space="preserve">10087 </t>
+          <t xml:space="preserve">10113 </t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -30373,12 +30373,12 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>CASTILLO 40</t>
+          <t>CONCORDIA 4213</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -30388,7 +30388,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>814108420</t>
+          <t>814111798</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -30398,7 +30398,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
@@ -30420,24 +30420,24 @@
         <v>1</v>
       </c>
       <c r="M350" t="n">
-        <v>-58.430621</v>
+        <v>-58.506878</v>
       </c>
       <c r="N350" t="n">
-        <v>-34.599429</v>
+        <v>-34.59474</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P350" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q350" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R350" t="inlineStr">
@@ -30449,7 +30449,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t xml:space="preserve">10102 </t>
+          <t xml:space="preserve">10119 </t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -30459,12 +30459,12 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>ELCANO AV. 3950</t>
+          <t>TRIUNVIRATO AV. 5900</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -30474,7 +30474,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>814108464</t>
+          <t>814111801</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -30499,21 +30499,21 @@
       </c>
       <c r="K351" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L351" t="n">
         <v>1</v>
       </c>
       <c r="M351" t="n">
-        <v>-58.460457</v>
+        <v>-58.496593</v>
       </c>
       <c r="N351" t="n">
-        <v>-34.582381</v>
+        <v>-34.563646</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P351" t="inlineStr">
@@ -30523,7 +30523,7 @@
       </c>
       <c r="Q351" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R351" t="inlineStr">
@@ -30535,7 +30535,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t xml:space="preserve">10113 </t>
+          <t xml:space="preserve">10126 </t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -30545,7 +30545,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>CONCORDIA 4213</t>
+          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -30558,11 +30558,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t>814111798</t>
-        </is>
-      </c>
+      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -30570,12 +30566,12 @@
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J352" t="inlineStr">
@@ -30592,14 +30588,14 @@
         <v>1</v>
       </c>
       <c r="M352" t="n">
-        <v>-58.506878</v>
+        <v>-58.482122</v>
       </c>
       <c r="N352" t="n">
-        <v>-34.59474</v>
+        <v>-34.570386</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P352" t="inlineStr">
@@ -30609,7 +30605,7 @@
       </c>
       <c r="Q352" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R352" t="inlineStr">
@@ -30621,7 +30617,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t xml:space="preserve">10119 </t>
+          <t xml:space="preserve">10133 </t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -30631,7 +30627,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5900</t>
+          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -30646,7 +30642,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>814111801</t>
+          <t>814108490</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -30656,7 +30652,7 @@
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -30671,17 +30667,17 @@
       </c>
       <c r="K353" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L353" t="n">
         <v>1</v>
       </c>
       <c r="M353" t="n">
-        <v>-58.496593</v>
+        <v>-58.453426</v>
       </c>
       <c r="N353" t="n">
-        <v>-34.563646</v>
+        <v>-34.600121</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -30695,7 +30691,7 @@
       </c>
       <c r="Q353" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
@@ -30707,7 +30703,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t xml:space="preserve">10126 </t>
+          <t xml:space="preserve">10136 </t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -30717,12 +30713,12 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
+          <t>REPETTO, NICOLAS, DR. 2118</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -30730,7 +30726,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr"/>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>814108495</t>
+        </is>
+      </c>
       <c r="G354" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -30738,12 +30738,12 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J354" t="inlineStr">
@@ -30760,14 +30760,14 @@
         <v>1</v>
       </c>
       <c r="M354" t="n">
-        <v>-58.482122</v>
+        <v>-58.456381</v>
       </c>
       <c r="N354" t="n">
-        <v>-34.570386</v>
+        <v>-34.60076</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P354" t="inlineStr">
@@ -30777,7 +30777,7 @@
       </c>
       <c r="Q354" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>NRA-G</t>
         </is>
       </c>
       <c r="R354" t="inlineStr">
@@ -30789,7 +30789,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t xml:space="preserve">10133 </t>
+          <t xml:space="preserve">10145 </t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -30799,7 +30799,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
+          <t>DONADO 2554</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -30814,7 +30814,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>814108490</t>
+          <t>814108500</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -30846,14 +30846,14 @@
         <v>1</v>
       </c>
       <c r="M355" t="n">
-        <v>-58.453426</v>
+        <v>-58.478634</v>
       </c>
       <c r="N355" t="n">
-        <v>-34.600121</v>
+        <v>-34.569063</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P355" t="inlineStr">
@@ -30863,7 +30863,7 @@
       </c>
       <c r="Q355" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R355" t="inlineStr">
@@ -30875,7 +30875,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t xml:space="preserve">10136 </t>
+          <t xml:space="preserve">10147 </t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -30885,12 +30885,12 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 2118</t>
+          <t>ROOSEVELT FRANKLIN D. 4336</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -30900,7 +30900,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>814108495</t>
+          <t>814111809</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -30910,7 +30910,7 @@
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
@@ -30925,21 +30925,21 @@
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L356" t="n">
         <v>1</v>
       </c>
       <c r="M356" t="n">
-        <v>-58.456381</v>
+        <v>-58.479316</v>
       </c>
       <c r="N356" t="n">
-        <v>-34.60076</v>
+        <v>-34.568762</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P356" t="inlineStr">
@@ -30949,7 +30949,7 @@
       </c>
       <c r="Q356" t="inlineStr">
         <is>
-          <t>NRA-G</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -30961,7 +30961,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t xml:space="preserve">10145 </t>
+          <t xml:space="preserve">10148 </t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -30971,7 +30971,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>DONADO 2554</t>
+          <t>ACHA, MARIANO, GRAL. 2595</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -30986,7 +30986,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>814108500</t>
+          <t>814108503</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -31018,10 +31018,10 @@
         <v>1</v>
       </c>
       <c r="M357" t="n">
-        <v>-58.478634</v>
+        <v>-58.479759</v>
       </c>
       <c r="N357" t="n">
-        <v>-34.569063</v>
+        <v>-34.569184</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -31047,22 +31047,22 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t xml:space="preserve">10147 </t>
+          <t>-785</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>ROOSEVELT FRANKLIN D. 4336</t>
+          <t>FOREST AV. 1167</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -31072,7 +31072,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>814111809</t>
+          <t>814125584</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -31082,7 +31082,7 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>columna doblada</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
@@ -31097,17 +31097,17 @@
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L358" t="n">
         <v>1</v>
       </c>
       <c r="M358" t="n">
-        <v>-58.479316</v>
+        <v>-58.459624</v>
       </c>
       <c r="N358" t="n">
-        <v>-34.568762</v>
+        <v>-34.578831</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -31121,7 +31121,7 @@
       </c>
       <c r="Q358" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>ATH-O</t>
         </is>
       </c>
       <c r="R358" t="inlineStr">
@@ -31133,22 +31133,22 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t xml:space="preserve">10148 </t>
+          <t>-788</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ACHA, MARIANO, GRAL. 2595</t>
+          <t>AZURDUY JUANA 2004</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -31158,7 +31158,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>814108503</t>
+          <t>814125587</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -31168,7 +31168,7 @@
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I359" t="inlineStr">
@@ -31190,14 +31190,14 @@
         <v>1</v>
       </c>
       <c r="M359" t="n">
-        <v>-58.479759</v>
+        <v>-58.463454</v>
       </c>
       <c r="N359" t="n">
-        <v>-34.569184</v>
+        <v>-34.548783</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P359" t="inlineStr">
@@ -31207,7 +31207,7 @@
       </c>
       <c r="Q359" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>BLO-R</t>
         </is>
       </c>
       <c r="R359" t="inlineStr">
@@ -31219,7 +31219,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>-785</t>
+          <t>-789</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -31229,7 +31229,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>FOREST AV. 1167</t>
+          <t>BALLIVIAN 2749</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -31244,7 +31244,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>814125584</t>
+          <t>814125594</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -31254,7 +31254,7 @@
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>columna doblada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
@@ -31276,14 +31276,14 @@
         <v>1</v>
       </c>
       <c r="M360" t="n">
-        <v>-58.459624</v>
+        <v>-58.481306</v>
       </c>
       <c r="N360" t="n">
-        <v>-34.578831</v>
+        <v>-34.581055</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P360" t="inlineStr">
@@ -31293,7 +31293,7 @@
       </c>
       <c r="Q360" t="inlineStr">
         <is>
-          <t>ATH-O</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -31305,7 +31305,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>-788</t>
+          <t>-790</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -31315,12 +31315,12 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>AZURDUY JUANA 2004</t>
+          <t>BAUNESS 2834</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -31330,7 +31330,7 @@
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>814125587</t>
+          <t>814125602</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -31362,14 +31362,14 @@
         <v>1</v>
       </c>
       <c r="M361" t="n">
-        <v>-58.463454</v>
+        <v>-58.490491</v>
       </c>
       <c r="N361" t="n">
-        <v>-34.548783</v>
+        <v>-34.571674</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P361" t="inlineStr">
@@ -31379,7 +31379,7 @@
       </c>
       <c r="Q361" t="inlineStr">
         <is>
-          <t>BLO-R</t>
+          <t>PUE-D</t>
         </is>
       </c>
       <c r="R361" t="inlineStr">
@@ -31391,7 +31391,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>-789</t>
+          <t>-791</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -31401,12 +31401,12 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>BALLIVIAN 2749</t>
+          <t>BLANCO ENCALADA 5264</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -31416,7 +31416,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>814125594</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -31426,7 +31426,7 @@
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t xml:space="preserve">correr </t>
         </is>
       </c>
       <c r="I362" t="inlineStr">
@@ -31436,7 +31436,7 @@
       </c>
       <c r="J362" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K362" t="inlineStr">
@@ -31448,10 +31448,10 @@
         <v>1</v>
       </c>
       <c r="M362" t="n">
-        <v>-58.481306</v>
+        <v>-58.48847</v>
       </c>
       <c r="N362" t="n">
-        <v>-34.581055</v>
+        <v>-34.576825</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -31465,7 +31465,7 @@
       </c>
       <c r="Q362" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R362" t="inlineStr">
@@ -31477,7 +31477,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>-790</t>
+          <t>-800</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -31487,7 +31487,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>BAUNESS 2834</t>
+          <t>ESTOMBA 1849</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -31502,7 +31502,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>814125602</t>
+          <t>814125637</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -31512,7 +31512,7 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
@@ -31534,14 +31534,14 @@
         <v>1</v>
       </c>
       <c r="M363" t="n">
-        <v>-58.490491</v>
+        <v>-58.469466</v>
       </c>
       <c r="N363" t="n">
-        <v>-34.571674</v>
+        <v>-34.572973</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P363" t="inlineStr">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="Q363" t="inlineStr">
         <is>
-          <t>PUE-D</t>
+          <t>ATH-A</t>
         </is>
       </c>
       <c r="R363" t="inlineStr">
@@ -31563,7 +31563,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>-791</t>
+          <t>-803</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -31573,12 +31573,12 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>BLANCO ENCALADA 5264</t>
+          <t>LA PAMPA 3810</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -31588,7 +31588,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125652</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t xml:space="preserve">correr </t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
@@ -31608,7 +31608,7 @@
       </c>
       <c r="J364" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
@@ -31620,14 +31620,14 @@
         <v>1</v>
       </c>
       <c r="M364" t="n">
-        <v>-58.48847</v>
+        <v>-58.468358</v>
       </c>
       <c r="N364" t="n">
-        <v>-34.576825</v>
+        <v>-34.573132</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P364" t="inlineStr">
@@ -31637,7 +31637,7 @@
       </c>
       <c r="Q364" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>ATH-A</t>
         </is>
       </c>
       <c r="R364" t="inlineStr">
@@ -31649,7 +31649,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>-800</t>
+          <t>-808</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -31659,7 +31659,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ESTOMBA 1849</t>
+          <t>MELIAN AV. 2716</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -31674,7 +31674,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>814125637</t>
+          <t>814125660</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -31706,10 +31706,10 @@
         <v>1</v>
       </c>
       <c r="M365" t="n">
-        <v>-58.469466</v>
+        <v>-58.473328</v>
       </c>
       <c r="N365" t="n">
-        <v>-34.572973</v>
+        <v>-34.563428</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -31723,7 +31723,7 @@
       </c>
       <c r="Q365" t="inlineStr">
         <is>
-          <t>ATH-A</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R365" t="inlineStr">
@@ -31735,7 +31735,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>-803</t>
+          <t>-809</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -31745,12 +31745,12 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>LA PAMPA 3810</t>
+          <t>MENDOZA 2122</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -31760,7 +31760,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>814125652</t>
+          <t>814125661</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -31792,14 +31792,14 @@
         <v>1</v>
       </c>
       <c r="M366" t="n">
-        <v>-58.468358</v>
+        <v>-58.454849</v>
       </c>
       <c r="N366" t="n">
-        <v>-34.573132</v>
+        <v>-34.559562</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P366" t="inlineStr">
@@ -31809,7 +31809,7 @@
       </c>
       <c r="Q366" t="inlineStr">
         <is>
-          <t>ATH-A</t>
+          <t>BLO-O</t>
         </is>
       </c>
       <c r="R366" t="inlineStr">
@@ -31821,7 +31821,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>-808</t>
+          <t>-813</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -31831,12 +31831,12 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>MELIAN AV. 2716</t>
+          <t>MURILLO 854</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -31846,7 +31846,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>814125660</t>
+          <t>814125670</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -31856,7 +31856,7 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>bae corroida</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -31878,14 +31878,14 @@
         <v>1</v>
       </c>
       <c r="M367" t="n">
-        <v>-58.473328</v>
+        <v>-58.445269</v>
       </c>
       <c r="N367" t="n">
-        <v>-34.563428</v>
+        <v>-34.599357</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P367" t="inlineStr">
@@ -31895,7 +31895,7 @@
       </c>
       <c r="Q367" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R367" t="inlineStr">
@@ -31907,7 +31907,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>-809</t>
+          <t>-814</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -31917,12 +31917,12 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>MENDOZA 2122</t>
+          <t>OLAZABAL AV. 4545</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -31932,7 +31932,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>814125661</t>
+          <t>814125673</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -31942,7 +31942,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -31964,14 +31964,14 @@
         <v>1</v>
       </c>
       <c r="M368" t="n">
-        <v>-58.454849</v>
+        <v>-58.480067</v>
       </c>
       <c r="N368" t="n">
-        <v>-34.559562</v>
+        <v>-34.573072</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P368" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="Q368" t="inlineStr">
         <is>
-          <t>BLO-O</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R368" t="inlineStr">
@@ -31993,7 +31993,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>-813</t>
+          <t>-815</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -32003,12 +32003,12 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>MURILLO 854</t>
+          <t>PESTALOZZI 3482</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -32018,7 +32018,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>814125670</t>
+          <t>814125676</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -32028,7 +32028,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>bae corroida</t>
+          <t>base podrida</t>
         </is>
       </c>
       <c r="I369" t="inlineStr">
@@ -32043,17 +32043,17 @@
       </c>
       <c r="K369" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L369" t="n">
         <v>1</v>
       </c>
       <c r="M369" t="n">
-        <v>-58.445269</v>
+        <v>-58.50075</v>
       </c>
       <c r="N369" t="n">
-        <v>-34.599357</v>
+        <v>-34.567798</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -32067,7 +32067,7 @@
       </c>
       <c r="Q369" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>PUE-H</t>
         </is>
       </c>
       <c r="R369" t="inlineStr">
@@ -32079,7 +32079,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>-814</t>
+          <t>-816</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -32089,7 +32089,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>OLAZABAL AV. 4545</t>
+          <t>PINTO 4609</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -32104,7 +32104,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>814125673</t>
+          <t>814125678</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -32136,14 +32136,14 @@
         <v>1</v>
       </c>
       <c r="M370" t="n">
-        <v>-58.480067</v>
+        <v>-58.481182</v>
       </c>
       <c r="N370" t="n">
-        <v>-34.573072</v>
+        <v>-34.544737</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P370" t="inlineStr">
@@ -32153,7 +32153,7 @@
       </c>
       <c r="Q370" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R370" t="inlineStr">
@@ -32165,22 +32165,22 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>-815</t>
+          <t>994PN</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>6/2/2026</t>
+          <t>6/5/2026</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>PESTALOZZI 3482</t>
+          <t>MARIANO ACHA 994</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -32190,7 +32190,7 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>814125676</t>
+          <t>814254408</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
@@ -32200,7 +32200,7 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>base podrida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -32215,21 +32215,21 @@
       </c>
       <c r="K371" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L371" t="n">
         <v>1</v>
       </c>
       <c r="M371" t="n">
-        <v>-58.50075</v>
+        <v>-58.472091</v>
       </c>
       <c r="N371" t="n">
-        <v>-34.567798</v>
+        <v>-34.583875</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P371" t="inlineStr">
@@ -32239,182 +32239,10 @@
       </c>
       <c r="Q371" t="inlineStr">
         <is>
-          <t>PUE-H</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R371" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" t="inlineStr">
-        <is>
-          <t>-816</t>
-        </is>
-      </c>
-      <c r="B372" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C372" t="inlineStr">
-        <is>
-          <t>PINTO 4609</t>
-        </is>
-      </c>
-      <c r="D372" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E372" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F372" t="inlineStr">
-        <is>
-          <t>814125678</t>
-        </is>
-      </c>
-      <c r="G372" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H372" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I372" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J372" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K372" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L372" t="n">
-        <v>1</v>
-      </c>
-      <c r="M372" t="n">
-        <v>-58.481182</v>
-      </c>
-      <c r="N372" t="n">
-        <v>-34.544737</v>
-      </c>
-      <c r="O372" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P372" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q372" t="inlineStr">
-        <is>
-          <t>COG-Q</t>
-        </is>
-      </c>
-      <c r="R372" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="inlineStr">
-        <is>
-          <t>994PN</t>
-        </is>
-      </c>
-      <c r="B373" t="inlineStr">
-        <is>
-          <t>6/5/2026</t>
-        </is>
-      </c>
-      <c r="C373" t="inlineStr">
-        <is>
-          <t>MARIANO ACHA 994</t>
-        </is>
-      </c>
-      <c r="D373" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E373" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F373" t="inlineStr">
-        <is>
-          <t>814254408</t>
-        </is>
-      </c>
-      <c r="G373" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H373" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I373" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J373" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K373" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L373" t="n">
-        <v>1</v>
-      </c>
-      <c r="M373" t="n">
-        <v>-58.472091</v>
-      </c>
-      <c r="N373" t="n">
-        <v>-34.583875</v>
-      </c>
-      <c r="O373" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P373" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q373" t="inlineStr">
-        <is>
-          <t>ATH-F</t>
-        </is>
-      </c>
-      <c r="R373" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-29 12:39:09)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R177"/>
+  <dimension ref="A1:R176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13391,7 +13391,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">9970 </t>
+          <t xml:space="preserve">9971 </t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ECHEVERRIA 5051</t>
+          <t>ECHEVERRIA 5021</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -13416,7 +13416,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>814111395</t>
+          <t>814111401</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -13448,10 +13448,10 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.481099</v>
+        <v>-58.480634</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.578912</v>
+        <v>-34.578647</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -13477,7 +13477,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">9971 </t>
+          <t xml:space="preserve">9993 </t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -13487,7 +13487,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ECHEVERRIA 5021</t>
+          <t>MONROE 5212</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -13502,7 +13502,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>814111401</t>
+          <t>814111591</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -13534,10 +13534,10 @@
         <v>1</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.480634</v>
+        <v>-58.487529</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.578647</v>
+        <v>-34.575028</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -13563,7 +13563,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">9993 </t>
+          <t xml:space="preserve">9996 </t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -13573,7 +13573,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>MONROE 5212</t>
+          <t>ZAMUDIO 4784</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -13588,7 +13588,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>814111591</t>
+          <t>814111621</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -13620,10 +13620,10 @@
         <v>1</v>
       </c>
       <c r="M154" t="n">
-        <v>-58.487529</v>
+        <v>-58.497199</v>
       </c>
       <c r="N154" t="n">
-        <v>-34.575028</v>
+        <v>-34.582097</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>PUE-M</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -13649,17 +13649,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">9996 </t>
+          <t xml:space="preserve">8962 </t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>ZAMUDIO 4784</t>
+          <t>CONGRESO AV. 5856</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -13674,7 +13674,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>814111621</t>
+          <t>814108043</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -13684,7 +13684,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -13706,10 +13706,10 @@
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>-58.497199</v>
+        <v>-58.499051</v>
       </c>
       <c r="N155" t="n">
-        <v>-34.582097</v>
+        <v>-34.57451</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -13723,7 +13723,7 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>PUE-M</t>
+          <t>PUE-I</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
@@ -13735,7 +13735,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">8962 </t>
+          <t xml:space="preserve">8982 </t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CONGRESO AV. 5856</t>
+          <t>LOPEZ, CARLOS ANTONIO 2197</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>814108043</t>
+          <t>814108057</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -13792,10 +13792,10 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-58.499051</v>
+        <v>-58.494928</v>
       </c>
       <c r="N156" t="n">
-        <v>-34.57451</v>
+        <v>-34.580378</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -13809,7 +13809,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>PUE-I</t>
+          <t>PUE-M</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13821,7 +13821,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">8982 </t>
+          <t xml:space="preserve">10024 </t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -13831,7 +13831,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>LOPEZ, CARLOS ANTONIO 2197</t>
+          <t>IBERA 6146</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -13846,7 +13846,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>814108057</t>
+          <t>814111657</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -13878,10 +13878,10 @@
         <v>1</v>
       </c>
       <c r="M157" t="n">
-        <v>-58.494928</v>
+        <v>-58.502338</v>
       </c>
       <c r="N157" t="n">
-        <v>-34.580378</v>
+        <v>-34.573275</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -13895,7 +13895,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>PUE-M</t>
+          <t>PUE-I</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -13907,7 +13907,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">10024 </t>
+          <t xml:space="preserve">10026 </t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>IBERA 6146</t>
+          <t>HUMBOLDT 47</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -13932,7 +13932,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>814111657</t>
+          <t>814111684</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -13964,10 +13964,10 @@
         <v>1</v>
       </c>
       <c r="M158" t="n">
-        <v>-58.502338</v>
+        <v>-58.451981</v>
       </c>
       <c r="N158" t="n">
-        <v>-34.573275</v>
+        <v>-34.597952</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -13981,7 +13981,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>PUE-I</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -13993,17 +13993,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">10026 </t>
+          <t xml:space="preserve">10027 </t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/7/2026</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>HUMBOLDT 47</t>
+          <t>HUMBOLDT 37</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -14018,7 +14018,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>814111684</t>
+          <t>814111686</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -14050,10 +14050,10 @@
         <v>1</v>
       </c>
       <c r="M159" t="n">
-        <v>-58.451981</v>
+        <v>-58.452157</v>
       </c>
       <c r="N159" t="n">
-        <v>-34.597952</v>
+        <v>-34.598081</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -14079,17 +14079,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">10027 </t>
+          <t xml:space="preserve">10060 </t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>5/7/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>HUMBOLDT 37</t>
+          <t xml:space="preserve">AREVALO 2951 </t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>814111686</t>
+          <t>814108282</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -14114,7 +14114,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -14136,24 +14136,24 @@
         <v>1</v>
       </c>
       <c r="M160" t="n">
-        <v>-58.452157</v>
+        <v>-58.430757</v>
       </c>
       <c r="N160" t="n">
-        <v>-34.598081</v>
+        <v>-34.571657</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14165,7 +14165,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">10060 </t>
+          <t xml:space="preserve">10070 </t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t xml:space="preserve">AREVALO 2951 </t>
+          <t>NUÑEZ 4634</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>814108282</t>
+          <t>814108373</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -14200,7 +14200,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -14222,24 +14222,24 @@
         <v>1</v>
       </c>
       <c r="M161" t="n">
-        <v>-58.430757</v>
+        <v>-58.487462</v>
       </c>
       <c r="N161" t="n">
-        <v>-34.571657</v>
+        <v>-34.561007</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14251,7 +14251,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">10070 </t>
+          <t xml:space="preserve">10084 </t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>NUÑEZ 4634</t>
+          <t>UGARTE, MANUEL 3258</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -14276,7 +14276,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>814108373</t>
+          <t>814108396</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -14308,14 +14308,14 @@
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>-58.487462</v>
+        <v>-58.470323</v>
       </c>
       <c r="N162" t="n">
-        <v>-34.561007</v>
+        <v>-34.560769</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -14337,7 +14337,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">10084 </t>
+          <t xml:space="preserve">10113 </t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>UGARTE, MANUEL 3258</t>
+          <t>CONCORDIA 4213</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>814108396</t>
+          <t>814111798</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -14372,7 +14372,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -14394,14 +14394,14 @@
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>-58.470323</v>
+        <v>-58.506878</v>
       </c>
       <c r="N163" t="n">
-        <v>-34.560769</v>
+        <v>-34.59474</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -14411,7 +14411,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -14423,7 +14423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">10113 </t>
+          <t xml:space="preserve">10126 </t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -14433,7 +14433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>CONCORDIA 4213</t>
+          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -14446,11 +14446,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>814111798</t>
-        </is>
-      </c>
+      <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -14458,12 +14454,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -14480,14 +14476,14 @@
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>-58.506878</v>
+        <v>-58.482122</v>
       </c>
       <c r="N164" t="n">
-        <v>-34.59474</v>
+        <v>-34.570386</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -14497,7 +14493,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -14509,7 +14505,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">10126 </t>
+          <t xml:space="preserve">10133 </t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -14519,7 +14515,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
+          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -14532,7 +14528,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>814108490</t>
+        </is>
+      </c>
       <c r="G165" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -14540,12 +14540,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -14562,14 +14562,14 @@
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.482122</v>
+        <v>-58.453426</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.570386</v>
+        <v>-34.600121</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -14579,7 +14579,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14591,7 +14591,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">10133 </t>
+          <t xml:space="preserve">10145 </t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
+          <t>DONADO 2554</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -14616,7 +14616,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>814108490</t>
+          <t>814108500</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -14648,14 +14648,14 @@
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.453426</v>
+        <v>-58.478634</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.600121</v>
+        <v>-34.569063</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
@@ -14665,7 +14665,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -14677,7 +14677,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">10145 </t>
+          <t xml:space="preserve">10147 </t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>DONADO 2554</t>
+          <t>ROOSEVELT FRANKLIN D. 4336</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>814108500</t>
+          <t>814111809</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -14727,17 +14727,17 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L167" t="n">
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.478634</v>
+        <v>-58.479316</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.569063</v>
+        <v>-34.568762</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -14763,7 +14763,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">10147 </t>
+          <t xml:space="preserve">10148 </t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ROOSEVELT FRANKLIN D. 4336</t>
+          <t>ACHA, MARIANO, GRAL. 2595</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>814111809</t>
+          <t>814108503</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -14813,17 +14813,17 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L168" t="n">
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.479316</v>
+        <v>-58.479759</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.568762</v>
+        <v>-34.569184</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -14849,22 +14849,22 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">10148 </t>
+          <t>-788</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ACHA, MARIANO, GRAL. 2595</t>
+          <t>AZURDUY JUANA 2004</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>814108503</t>
+          <t>814125587</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -14884,7 +14884,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -14906,14 +14906,14 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>-58.479759</v>
+        <v>-58.463454</v>
       </c>
       <c r="N169" t="n">
-        <v>-34.569184</v>
+        <v>-34.548783</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
@@ -14923,7 +14923,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>BLO-R</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -14935,7 +14935,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>-788</t>
+          <t>-790</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -14945,12 +14945,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AZURDUY JUANA 2004</t>
+          <t>BAUNESS 2834</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -14960,7 +14960,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>814125587</t>
+          <t>814125602</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -14992,14 +14992,14 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.463454</v>
+        <v>-58.490491</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.548783</v>
+        <v>-34.571674</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>BLO-R</t>
+          <t>PUE-D</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -15021,7 +15021,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>-790</t>
+          <t>-791</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>BAUNESS 2834</t>
+          <t>BLANCO ENCALADA 5264</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>814125602</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t xml:space="preserve">correr </t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -15078,10 +15078,10 @@
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>-58.490491</v>
+        <v>-58.48847</v>
       </c>
       <c r="N171" t="n">
-        <v>-34.571674</v>
+        <v>-34.576825</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -15095,7 +15095,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>PUE-D</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15107,7 +15107,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>-791</t>
+          <t>-800</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -15117,7 +15117,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>BLANCO ENCALADA 5264</t>
+          <t>ESTOMBA 1849</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125637</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t xml:space="preserve">correr </t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -15152,7 +15152,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -15164,14 +15164,14 @@
         <v>1</v>
       </c>
       <c r="M172" t="n">
-        <v>-58.48847</v>
+        <v>-58.469466</v>
       </c>
       <c r="N172" t="n">
-        <v>-34.576825</v>
+        <v>-34.572973</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P172" t="inlineStr">
@@ -15181,7 +15181,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>ATH-A</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15193,7 +15193,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>-800</t>
+          <t>-808</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>ESTOMBA 1849</t>
+          <t>MELIAN AV. 2716</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>814125637</t>
+          <t>814125660</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -15250,10 +15250,10 @@
         <v>1</v>
       </c>
       <c r="M173" t="n">
-        <v>-58.469466</v>
+        <v>-58.473328</v>
       </c>
       <c r="N173" t="n">
-        <v>-34.572973</v>
+        <v>-34.563428</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -15267,7 +15267,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>ATH-A</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -15279,7 +15279,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>-808</t>
+          <t>-809</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -15289,12 +15289,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>MELIAN AV. 2716</t>
+          <t>MENDOZA 2122</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -15304,7 +15304,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>814125660</t>
+          <t>814125661</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -15336,14 +15336,14 @@
         <v>1</v>
       </c>
       <c r="M174" t="n">
-        <v>-58.473328</v>
+        <v>-58.454849</v>
       </c>
       <c r="N174" t="n">
-        <v>-34.563428</v>
+        <v>-34.559562</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P174" t="inlineStr">
@@ -15353,7 +15353,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>BLO-O</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -15365,7 +15365,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>-809</t>
+          <t>-814</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -15375,12 +15375,12 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>MENDOZA 2122</t>
+          <t>OLAZABAL AV. 4545</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -15390,7 +15390,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>814125661</t>
+          <t>814125673</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -15400,7 +15400,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -15422,14 +15422,14 @@
         <v>1</v>
       </c>
       <c r="M175" t="n">
-        <v>-58.454849</v>
+        <v>-58.480067</v>
       </c>
       <c r="N175" t="n">
-        <v>-34.559562</v>
+        <v>-34.573072</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
@@ -15439,7 +15439,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>BLO-O</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -15451,7 +15451,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>-814</t>
+          <t>-816</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -15461,7 +15461,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>OLAZABAL AV. 4545</t>
+          <t>PINTO 4609</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -15476,7 +15476,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>814125673</t>
+          <t>814125678</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -15508,14 +15508,14 @@
         <v>1</v>
       </c>
       <c r="M176" t="n">
-        <v>-58.480067</v>
+        <v>-58.481182</v>
       </c>
       <c r="N176" t="n">
-        <v>-34.573072</v>
+        <v>-34.544737</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P176" t="inlineStr">
@@ -15525,96 +15525,10 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>-816</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>PINTO 4609</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>814125678</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L177" t="n">
-        <v>1</v>
-      </c>
-      <c r="M177" t="n">
-        <v>-58.481182</v>
-      </c>
-      <c r="N177" t="n">
-        <v>-34.544737</v>
-      </c>
-      <c r="O177" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P177" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q177" t="inlineStr">
-        <is>
-          <t>COG-Q</t>
-        </is>
-      </c>
-      <c r="R177" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-07-02 12:18:46)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_NEW.xlsx
+++ b/mapa_interactivo_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R176"/>
+  <dimension ref="A1:R173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2395,7 +2395,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-365</t>
+          <t>7966</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>QUESADA /ALT/ 5290</t>
+          <t>QUESADA /ALT/ 6088</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>804839995</t>
+          <t>804840016</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Columna nueva de PVC fuera de plomo.  - VIRARDI</t>
+          <t>Aplomar columna de 168 cambiar rienda.  - VIRARDI</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2452,10 +2452,10 @@
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.491934</v>
+        <v>-58.501418</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.569348</v>
+        <v>-34.574363</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PUE-I</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2481,22 +2481,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7966</t>
+          <t>5624</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4/14/2025</t>
+          <t>4/22/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>QUESADA /ALT/ 6088</t>
+          <t>PINO, VIRREY DEL 3456</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>804840016</t>
+          <t>804876043</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2516,12 +2516,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Aplomar columna de 168 cambiar rienda.  - VIRARDI</t>
+          <t>Desmonte de poste</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2531,21 +2531,21 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.501418</v>
+        <v>-58.464354</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.574363</v>
+        <v>-34.572486</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PUE-I</t>
+          <t>ATH-R</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5624</t>
+          <t>-368</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PINO, VIRREY DEL 3456</t>
+          <t>ARIAS /ALT/ 1620</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>804876043</t>
+          <t>804876039</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2602,12 +2602,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Desmonte de poste</t>
+          <t xml:space="preserve">Aplomar columna 168 con rienda </t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2617,21 +2617,21 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.464354</v>
+        <v>-58.465608</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.572486</v>
+        <v>-34.538489</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>ATH-R</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2653,17 +2653,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>-368</t>
+          <t>804922171</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4/22/2025</t>
+          <t>4/24/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ARIAS /ALT/ 1620</t>
+          <t>Virrey Arredondo 3581</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>804876039</t>
+          <t>804922171</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aplomar columna 168 con rienda </t>
+          <t>Aplomar</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2710,14 +2710,14 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.465608</v>
+        <v>-58.459513</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.538489</v>
+        <v>-34.578019</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>ATH-O</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2739,17 +2739,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>804922171</t>
+          <t>805507192</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4/24/2025</t>
+          <t>4/28/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Virrey Arredondo 3581</t>
+          <t>Virrey Arredondo 2821</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>804922171</t>
+          <t>805507192</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2774,12 +2774,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2796,10 +2796,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.459513</v>
+        <v>-58.454065</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.578019</v>
+        <v>-34.57105</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>ATH-O</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2825,17 +2825,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>805507192</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>4/28/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Virrey Arredondo 2821</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2845,12 +2845,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>805507192</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2870,22 +2870,22 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.454065</v>
+        <v>-58.451835</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.57105</v>
+        <v>-34.562646</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2911,7 +2911,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>-408</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>Larralde 2847</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>805791941</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2946,17 +2946,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Aplomar columna 114</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2968,14 +2968,14 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.451835</v>
+        <v>-58.472267</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.562646</v>
+        <v>-34.551163</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>COG-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2997,22 +2997,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>-408</t>
+          <t>-421</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>5/26/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Larralde 2847</t>
+          <t>BESARES 1699</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>805791941</t>
+          <t>806926565</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3032,17 +3032,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Aplomar columna 114</t>
+          <t>Cambiar columna 114 picada en base tener en cuenta que hay acometidas subterraneas que bajan por la columna para entrar en Libertador 8008 tanto de HFC como FTTH colocar medias cañas y colocar cerca para que quedan precintadas a la columna</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3054,10 +3054,10 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.472267</v>
+        <v>-58.464144</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.551163</v>
+        <v>-34.541832</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>COG-M</t>
+          <t>BLO-F</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>-421</t>
+          <t>5885</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BESARES 1699</t>
+          <t>CABILDO AV. 1500</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>806926565</t>
+          <t>806944768</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base tener en cuenta que hay acometidas subterraneas que bajan por la columna para entrar en Libertador 8008 tanto de HFC como FTTH colocar medias cañas y colocar cerca para que quedan precintadas a la columna</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3140,14 +3140,14 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.464144</v>
+        <v>-58.450724</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.541832</v>
+        <v>-34.567086</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>BLO-F</t>
+          <t>COG-D</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3169,7 +3169,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5885</t>
+          <t>5883</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CABILDO AV. 1500</t>
+          <t>CONGRESO AV. 2699</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>806944768</t>
+          <t>806944763</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3226,14 +3226,14 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.450724</v>
+        <v>-58.46522</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.567086</v>
+        <v>-34.556786</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>COG-D</t>
+          <t>COG-K</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3255,22 +3255,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5883</t>
+          <t>5935</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>5/26/2025</t>
+          <t>5/27/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CONGRESO AV. 2699</t>
+          <t>ALVAREZ THOMAS AV. 3305</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>806944763</t>
+          <t>807044131</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3290,12 +3290,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna inclinada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3305,21 +3305,21 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.46522</v>
+        <v>-58.483927</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.556786</v>
+        <v>-34.570689</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>COG-K</t>
+          <t>PUE-E</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3341,22 +3341,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5935</t>
+          <t>807044200</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>5/27/2025</t>
+          <t>5/29/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 3305</t>
+          <t>11 de Septiembre de 1888 4662</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>807044131</t>
+          <t>807044200</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Columna inclinada</t>
+          <t>CAMBIAR COLUMNA MUY INCLINADA POR POSTE PRFV 400, COLOCAR A 40 CMTS DEL CORDON</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3398,14 +3398,14 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.483927</v>
+        <v>-58.467458</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.570689</v>
+        <v>-34.537549</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>PUE-E</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3427,17 +3427,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>807044200</t>
+          <t>8928</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>5/29/2025</t>
+          <t>6/4/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>11 de Septiembre de 1888 4662</t>
+          <t>General Enrique Martinez 188</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>807044200</t>
+          <t>807168186</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3462,12 +3462,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA MUY INCLINADA POR POSTE PRFV 400, COLOCAR A 40 CMTS DEL CORDON</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3477,31 +3477,31 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.467458</v>
+        <v>-58.446125</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.537549</v>
+        <v>-34.580819</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3513,7 +3513,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8928</t>
+          <t>-469</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>General Enrique Martinez 188</t>
+          <t>Newbery 3323</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>807168186</t>
+          <t>800966689</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3563,17 +3563,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.446125</v>
+        <v>-58.447732</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.580819</v>
+        <v>-34.580408</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3599,17 +3599,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>-469</t>
+          <t>6229</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>6/4/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Newbery 3323</t>
+          <t>ALVAREZ THOMAS AV. 309</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>800966689</t>
+          <t>807762987</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t xml:space="preserve">Reparar rienda </t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3656,10 +3656,10 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.447732</v>
+        <v>-58.44848</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.580408</v>
+        <v>-34.581338</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6229</t>
+          <t>-488</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3695,12 +3695,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 309</t>
+          <t>Blanco Encalada 4896</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>807762987</t>
+          <t>807763099</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3720,12 +3720,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reparar rienda </t>
+          <t>Pendiente traspaso rxo y retiro de columna podrida</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3735,31 +3735,31 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.44848</v>
+        <v>-58.484729</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.581338</v>
+        <v>-34.574614</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3771,22 +3771,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>-488</t>
+          <t>6506</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>7/10/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Blanco Encalada 4896</t>
+          <t>Ohiggins 1611</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>807763099</t>
+          <t>808148679</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Pendiente traspaso rxo y retiro de columna podrida</t>
+          <t>Columna podrida en la base</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3816,26 +3816,26 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.484729</v>
+        <v>-58.448993</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.574614</v>
+        <v>-34.564383</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3857,22 +3857,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>6506</t>
+          <t>-507</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>7/10/2025</t>
+          <t>7/14/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ohiggins 1611</t>
+          <t>Tamborini 3291</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>808148679</t>
+          <t>808194229</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Columna podrida en la base</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3914,14 +3914,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.448993</v>
+        <v>-58.473937</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.564383</v>
+        <v>-34.557355</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3943,7 +3943,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>-507</t>
+          <t>-508</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Tamborini 3291</t>
+          <t>Moldes 2463</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>808194229</t>
+          <t>808194234</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -4000,10 +4000,10 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.473937</v>
+        <v>-58.462281</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.557355</v>
+        <v>-34.560321</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -4017,7 +4017,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>COG-J</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4029,17 +4029,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>-508</t>
+          <t>-546</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>7/14/2025</t>
+          <t>8/5/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Moldes 2463</t>
+          <t>Albarellos 3031</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>808194234</t>
+          <t>808720857</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -4086,14 +4086,14 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.462281</v>
+        <v>-58.511732</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.560321</v>
+        <v>-34.578688</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>COG-J</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4115,22 +4115,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>-546</t>
+          <t>6943</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>8/5/2025</t>
+          <t>8/14/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Albarellos 3031</t>
+          <t>SUPERI 1459</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>808720857</t>
+          <t>808972965</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4150,12 +4150,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Poste con base quebrada ver si es posible desmonte</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4165,21 +4165,21 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L44" t="n">
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.511732</v>
+        <v>-58.460834</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.578688</v>
+        <v>-34.573753</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4201,17 +4201,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6943</t>
+          <t>-559</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>8/14/2025</t>
+          <t>8/21/2025</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SUPERI 1459</t>
+          <t>Av. Del Libertador 6736</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>808972965</t>
+          <t>809098713</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Poste con base quebrada ver si es posible desmonte</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4251,21 +4251,21 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.460834</v>
+        <v>-58.453398</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.573753</v>
+        <v>-34.550238</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>BLO-E</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4287,22 +4287,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>-559</t>
+          <t>4166</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>8/21/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Av. Del Libertador 6736</t>
+          <t>ALTOLAGUIRRE 2201</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>809098713</t>
+          <t>809309591</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4344,14 +4344,14 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.453398</v>
+        <v>-58.489622</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.550238</v>
+        <v>-34.578426</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>BLO-E</t>
+          <t>PUE-C</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4373,17 +4373,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>4166</t>
+          <t>7111</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>9/1/2025</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ALTOLAGUIRRE 2201</t>
+          <t>VILELA 3699</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>809309591</t>
+          <t>809371823</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t xml:space="preserve">Cambiar </t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4423,21 +4423,21 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.489622</v>
+        <v>-58.482817</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.578426</v>
+        <v>-34.550845</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>PUE-C</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4459,17 +4459,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7111</t>
+          <t>7120</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>9/1/2025</t>
+          <t>9/2/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>VILELA 3699</t>
+          <t>BLANCO ENCALADA 4210</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>809371823</t>
+          <t>ICD30461848</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cambiar </t>
+          <t>Colocar R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4504,26 +4504,26 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.482817</v>
+        <v>-58.477593</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.550845</v>
+        <v>-34.570321</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4545,7 +4545,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7120</t>
+          <t>-579</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4555,12 +4555,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BLANCO ENCALADA 4210</t>
+          <t>Pedro Rivera 2546</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>ICD30461848</t>
+          <t>ICD30612785</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Colocar R400 para pedir traspaso de fuente</t>
+          <t>Colocar R200 para pedir traspaso de equipos</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -4602,14 +4602,14 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.477593</v>
+        <v>-58.462479</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.570321</v>
+        <v>-34.55765</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>COG-K</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4631,17 +4631,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>-579</t>
+          <t>-593</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>9/2/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Pedro Rivera 2546</t>
+          <t>HUSARES 2250</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ICD30612785</t>
+          <t>813350488</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Colocar R200 para pedir traspaso de equipos</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -4688,10 +4688,10 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.462479</v>
+        <v>-58.443269</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.55765</v>
+        <v>-34.552209</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>COG-K</t>
+          <t>BLO-B</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4717,7 +4717,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>-593</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HUSARES 2250</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>813350488</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4774,14 +4774,14 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.443269</v>
+        <v>-58.458298</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.552209</v>
+        <v>-34.566511</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>BLO-B</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4803,17 +4803,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>7225</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>9/16/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>AMENABAR 3590</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4828,7 +4828,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>809784519</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Reparar rienda y tambien reclaman columna picada pero no se ve la foto verificarla y evaluar cambio</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4853,21 +4853,21 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.458298</v>
+        <v>-58.470045</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.566511</v>
+        <v>-34.550272</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>COG-M</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4889,22 +4889,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>7225</t>
+          <t>S01186963</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>9/16/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AMENABAR 3590</t>
+          <t>WASHINGTON 4273</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>809784519</t>
+          <t>809800217</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Reparar rienda y tambien reclaman columna picada pero no se ve la foto verificarla y evaluar cambio</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4939,17 +4939,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.470045</v>
+        <v>-58.484798</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.550272</v>
+        <v>-34.550226</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>COG-M</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4975,17 +4975,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S01186963</t>
+          <t>2711</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>WASHINGTON 4273</t>
+          <t>RUIZ HUIDOBRO 3620</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>809800217</t>
+          <t>ICD30934235</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5010,12 +5010,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Trapaso de redes y desmonte</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5032,10 +5032,10 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.484798</v>
+        <v>-58.484082</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.550226</v>
+        <v>-34.549702</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -5061,22 +5061,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2711</t>
+          <t>-609</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>9/24/2025</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RUIZ HUIDOBRO 3620</t>
+          <t>Mcal Sucre 1837</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>ICD30934235</t>
+          <t>809972763</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5096,12 +5096,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Trapaso de redes y desmonte</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5118,14 +5118,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.484082</v>
+        <v>-58.449934</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.549702</v>
+        <v>-34.560847</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>-609</t>
+          <t>-610</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Mcal Sucre 1837</t>
+          <t>Mcal Sucre 1897</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>809972763</t>
+          <t>809972767</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5204,10 +5204,10 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.449934</v>
+        <v>-58.450295</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.560847</v>
+        <v>-34.561061</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5233,22 +5233,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>-610</t>
+          <t>7317</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>9/24/2025</t>
+          <t>9/25/2025</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Mcal Sucre 1897</t>
+          <t>MARMOL JOSE 588</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>809972767</t>
+          <t>809979740</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5290,24 +5290,24 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.450295</v>
+        <v>-58.425357</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.561061</v>
+        <v>-34.620223</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>ALM-B</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -7809,17 +7809,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>S00021988</t>
+          <t>S01337226</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>2/6/2026</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 1115</t>
+          <t>MOLDES 3055</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>811626996</t>
+          <t>811627125</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -7866,14 +7866,14 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.457565</v>
+        <v>-58.466692</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.578379</v>
+        <v>-34.555283</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>ATH-O</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7895,7 +7895,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>S01337226</t>
+          <t>S01375612</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>MOLDES 3055</t>
+          <t>LACROZE, FEDERICO AV. 2834</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>811627125</t>
+          <t>811627118</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -7930,7 +7930,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroidaq</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -7952,24 +7952,24 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.466692</v>
+        <v>-58.447177</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.555283</v>
+        <v>-34.574158</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7981,22 +7981,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>S01375612</t>
+          <t>8378</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2/6/2026</t>
+          <t>2/19/2026</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 2834</t>
+          <t>ANDONAEGUI 2383</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>811627118</t>
+          <t>812440211</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>corroidaq</t>
+          <t>base corroida inclinada</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -8038,24 +8038,24 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.447177</v>
+        <v>-58.489606</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.574158</v>
+        <v>-34.57655</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8067,7 +8067,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>8378</t>
+          <t>8386</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -8077,7 +8077,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ANDONAEGUI 2383</t>
+          <t>CRAMER 4262</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>812440211</t>
+          <t>812440206</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -8124,14 +8124,14 @@
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.489606</v>
+        <v>-58.476168</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.57655</v>
+        <v>-34.545546</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8153,17 +8153,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>8386</t>
+          <t>-750</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2/19/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CRAMER 4262</t>
+          <t>JURAMENTO 4979</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>812440206</t>
+          <t>812440599</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>base corroida inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -8210,14 +8210,14 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.476168</v>
+        <v>-58.481188</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.545546</v>
+        <v>-34.577198</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8239,7 +8239,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>-750</t>
+          <t>-754</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -8249,12 +8249,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>JURAMENTO 4979</t>
+          <t>PINO, VIRREY DEL 1503</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>812440599</t>
+          <t>812440515</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8296,14 +8296,14 @@
         <v>1</v>
       </c>
       <c r="M92" t="n">
-        <v>-58.481188</v>
+        <v>-58.442723</v>
       </c>
       <c r="N92" t="n">
-        <v>-34.577198</v>
+        <v>-34.56085</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
@@ -8313,7 +8313,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>BLO-A</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8325,7 +8325,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>-754</t>
+          <t>-761</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -8335,7 +8335,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>PINO, VIRREY DEL 1503</t>
+          <t>MOLDES 2901</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8350,7 +8350,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>812440515</t>
+          <t>812440341</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -8382,10 +8382,10 @@
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.442723</v>
+        <v>-58.465305</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.56085</v>
+        <v>-34.556794</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -8399,7 +8399,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>BLO-A</t>
+          <t>COG-K</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8411,17 +8411,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>-761</t>
+          <t>-769</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/2/2026</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MOLDES 2901</t>
+          <t>RIVERA, PEDRO I., DR. 2734</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>812440341</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -8446,7 +8446,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -8468,10 +8468,10 @@
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.465305</v>
+        <v>-58.464354</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.556794</v>
+        <v>-34.5587</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -8497,22 +8497,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>-769</t>
+          <t xml:space="preserve">8574 </t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>3/2/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>RIVERA, PEDRO I., DR. 2734</t>
+          <t xml:space="preserve">MANZANARES 4746 </t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Pendiente ADM OT GxC</t>
+          <t>812878883</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -8532,17 +8532,17 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -8554,10 +8554,10 @@
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.464354</v>
+        <v>-58.490797</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.5587</v>
+        <v>-34.558302</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -8571,7 +8571,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>COG-K</t>
+          <t>COG-O</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8583,17 +8583,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">8574 </t>
+          <t>9110</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/19/2026</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANZANARES 4746 </t>
+          <t>BESARES 3453</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>812878883</t>
+          <t>812879885</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -8618,12 +8618,12 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Columna Inclinada</t>
+          <t>Cambiar Poste por Columna</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -8640,10 +8640,10 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.490797</v>
+        <v>-58.48116</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.558302</v>
+        <v>-34.549119</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>COG-O</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8669,17 +8669,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>9110</t>
+          <t>8671</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>BESARES 3453</t>
+          <t>TRONADOR 284</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>812879885</t>
+          <t>812880206</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -8704,12 +8704,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Cambiar Poste por Columna</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -8726,14 +8726,14 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.48116</v>
+        <v>-58.470504</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.549119</v>
+        <v>-34.588131</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8743,7 +8743,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8755,7 +8755,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>8671</t>
+          <t>8676</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>TRONADOR 284</t>
+          <t>HOLMBERG 979</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>812880206</t>
+          <t>812880241</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8812,14 +8812,14 @@
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.470504</v>
+        <v>-58.468449</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.588131</v>
+        <v>-34.582898</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8841,7 +8841,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>8676</t>
+          <t>00289536</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>HOLMBERG 979</t>
+          <t>VALDENEGRO 3554</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8866,7 +8866,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>812880241</t>
+          <t>812880608</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -8876,12 +8876,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -8898,14 +8898,14 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.468449</v>
+        <v>-58.490576</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.582898</v>
+        <v>-34.561508</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8927,17 +8927,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>00289536</t>
+          <t>8647</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/24/2026</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>VALDENEGRO 3554</t>
+          <t xml:space="preserve">MELIAN AV 4827 </t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8952,7 +8952,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>812880608</t>
+          <t>812880706</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -8962,7 +8962,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -8984,10 +8984,10 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.490576</v>
+        <v>-58.487048</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.561508</v>
+        <v>-34.545509</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9013,22 +9013,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>8647</t>
+          <t>S00363991</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>3/24/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">MELIAN AV 4827 </t>
+          <t>ARCOS 2981</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9038,7 +9038,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>812880706</t>
+          <t>813046774</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -9048,7 +9048,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -9070,10 +9070,10 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.487048</v>
+        <v>-58.461029</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.545509</v>
+        <v>-34.552021</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -9087,7 +9087,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>COG-Q</t>
+          <t>BLO-Q</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9099,7 +9099,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>S00363991</t>
+          <t>8846</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -9109,12 +9109,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ARCOS 2981</t>
+          <t>RIVADAVIA AV 4245</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>813046774</t>
+          <t>813046970</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -9156,24 +9156,24 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.461029</v>
+        <v>-58.425567</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.552021</v>
+        <v>-34.613382</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>BLO-Q</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -13907,17 +13907,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">10026 </t>
+          <t xml:space="preserve">10027 </t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/7/2026</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>HUMBOLDT 47</t>
+          <t>HUMBOLDT 37</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -13932,7 +13932,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>814111684</t>
+          <t>814111686</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -13964,10 +13964,10 @@
         <v>1</v>
       </c>
       <c r="M158" t="n">
-        <v>-58.451981</v>
+        <v>-58.452157</v>
       </c>
       <c r="N158" t="n">
-        <v>-34.597952</v>
+        <v>-34.598081</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -13993,17 +13993,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">10027 </t>
+          <t xml:space="preserve">10060 </t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>5/7/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>HUMBOLDT 37</t>
+          <t xml:space="preserve">AREVALO 2951 </t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -14018,7 +14018,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>814111686</t>
+          <t>814108282</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -14050,24 +14050,24 @@
         <v>1</v>
       </c>
       <c r="M159" t="n">
-        <v>-58.452157</v>
+        <v>-58.430757</v>
       </c>
       <c r="N159" t="n">
-        <v>-34.598081</v>
+        <v>-34.571657</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14079,7 +14079,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">10060 </t>
+          <t xml:space="preserve">10070 </t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -14089,7 +14089,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t xml:space="preserve">AREVALO 2951 </t>
+          <t>NUÑEZ 4634</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>814108282</t>
+          <t>814108373</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -14114,7 +14114,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y VER POSIBILIDAD DE COLOCAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -14136,24 +14136,24 @@
         <v>1</v>
       </c>
       <c r="M160" t="n">
-        <v>-58.430757</v>
+        <v>-58.487462</v>
       </c>
       <c r="N160" t="n">
-        <v>-34.571657</v>
+        <v>-34.561007</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14165,7 +14165,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">10070 </t>
+          <t xml:space="preserve">10084 </t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>NUÑEZ 4634</t>
+          <t>UGARTE, MANUEL 3258</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>814108373</t>
+          <t>814108396</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -14222,14 +14222,14 @@
         <v>1</v>
       </c>
       <c r="M161" t="n">
-        <v>-58.487462</v>
+        <v>-58.470323</v>
       </c>
       <c r="N161" t="n">
-        <v>-34.561007</v>
+        <v>-34.560769</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
@@ -14239,7 +14239,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>COG-I</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14251,7 +14251,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">10084 </t>
+          <t xml:space="preserve">10113 </t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>UGARTE, MANUEL 3258</t>
+          <t>CONCORDIA 4213</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -14276,7 +14276,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>814108396</t>
+          <t>814111798</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -14308,14 +14308,14 @@
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>-58.470323</v>
+        <v>-58.506878</v>
       </c>
       <c r="N162" t="n">
-        <v>-34.560769</v>
+        <v>-34.59474</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -14337,7 +14337,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">10113 </t>
+          <t xml:space="preserve">10126 </t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>CONCORDIA 4213</t>
+          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -14360,11 +14360,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>814111798</t>
-        </is>
-      </c>
+      <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -14372,12 +14368,12 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -14394,14 +14390,14 @@
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>-58.506878</v>
+        <v>-58.482122</v>
       </c>
       <c r="N163" t="n">
-        <v>-34.59474</v>
+        <v>-34.570386</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -14411,7 +14407,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -14423,7 +14419,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">10126 </t>
+          <t xml:space="preserve">10133 </t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -14433,7 +14429,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROOSEVELT FRANKLIN D. 4647 </t>
+          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -14446,7 +14442,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>814108490</t>
+        </is>
+      </c>
       <c r="G164" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -14454,12 +14454,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -14476,14 +14476,14 @@
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>-58.482122</v>
+        <v>-58.453426</v>
       </c>
       <c r="N164" t="n">
-        <v>-34.570386</v>
+        <v>-34.600121</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -14493,7 +14493,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -14505,7 +14505,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">10133 </t>
+          <t xml:space="preserve">10145 </t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATALLA DEL PARI 593 </t>
+          <t>DONADO 2554</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -14530,7 +14530,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>814108490</t>
+          <t>814108500</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -14562,14 +14562,14 @@
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.453426</v>
+        <v>-58.478634</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.600121</v>
+        <v>-34.569063</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -14579,7 +14579,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14591,7 +14591,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">10145 </t>
+          <t xml:space="preserve">10147 </t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>DONADO 2554</t>
+          <t>ROOSEVELT FRANKLIN D. 4336</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -14616,7 +14616,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>814108500</t>
+          <t>814111809</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -14641,17 +14641,17 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L166" t="n">
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.478634</v>
+        <v>-58.479316</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.569063</v>
+        <v>-34.568762</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -14677,7 +14677,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">10147 </t>
+          <t xml:space="preserve">10148 </t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>ROOSEVELT FRANKLIN D. 4336</t>
+          <t>ACHA, MARIANO, GRAL. 2595</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>814111809</t>
+          <t>814108503</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -14727,17 +14727,17 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L167" t="n">
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.479316</v>
+        <v>-58.479759</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.568762</v>
+        <v>-34.569184</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -14763,22 +14763,22 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">10148 </t>
+          <t>-788</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ACHA, MARIANO, GRAL. 2595</t>
+          <t>AZURDUY JUANA 2004</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>814108503</t>
+          <t>814125587</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -14820,14 +14820,14 @@
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.479759</v>
+        <v>-58.463454</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.569184</v>
+        <v>-34.548783</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>BLO-R</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -14849,7 +14849,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>-788</t>
+          <t>-790</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -14859,12 +14859,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>AZURDUY JUANA 2004</t>
+          <t>BAUNESS 2834</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>814125587</t>
+          <t>814125602</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -14906,14 +14906,14 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>-58.463454</v>
+        <v>-58.490491</v>
       </c>
       <c r="N169" t="n">
-        <v>-34.548783</v>
+        <v>-34.571674</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
@@ -14923,7 +14923,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>BLO-R</t>
+          <t>PUE-D</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -14935,7 +14935,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>-790</t>
+          <t>-791</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>BAUNESS 2834</t>
+          <t>BLANCO ENCALADA 5264</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -14960,7 +14960,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>814125602</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -14970,7 +14970,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t xml:space="preserve">correr </t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -14980,7 +14980,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -14992,10 +14992,10 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.490491</v>
+        <v>-58.48847</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.571674</v>
+        <v>-34.576825</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -15009,7 +15009,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>PUE-D</t>
+          <t>ATH-C</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -15021,7 +15021,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>-791</t>
+          <t>-800</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>BLANCO ENCALADA 5264</t>
+          <t>ESTOMBA 1849</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125637</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t xml:space="preserve">correr </t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -15078,14 +15078,14 @@
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>-58.48847</v>
+        <v>-58.469466</v>
       </c>
       <c r="N171" t="n">
-        <v>-34.576825</v>
+        <v>-34.572973</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
@@ -15095,7 +15095,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>ATH-C</t>
+          <t>ATH-A</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15107,7 +15107,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>-800</t>
+          <t>-814</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -15117,7 +15117,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ESTOMBA 1849</t>
+          <t>OLAZABAL AV. 4545</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>814125637</t>
+          <t>814125673</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -15164,10 +15164,10 @@
         <v>1</v>
       </c>
       <c r="M172" t="n">
-        <v>-58.469466</v>
+        <v>-58.480067</v>
       </c>
       <c r="N172" t="n">
-        <v>-34.572973</v>
+        <v>-34.573072</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -15181,7 +15181,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>ATH-A</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15193,7 +15193,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>-808</t>
+          <t>-816</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>MELIAN AV. 2716</t>
+          <t>PINTO 4609</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>814125660</t>
+          <t>814125678</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -15250,14 +15250,14 @@
         <v>1</v>
       </c>
       <c r="M173" t="n">
-        <v>-58.473328</v>
+        <v>-58.481182</v>
       </c>
       <c r="N173" t="n">
-        <v>-34.563428</v>
+        <v>-34.544737</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P173" t="inlineStr">
@@ -15267,268 +15267,10 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>COG-I</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>-809</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>MENDOZA 2122</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>814125661</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L174" t="n">
-        <v>1</v>
-      </c>
-      <c r="M174" t="n">
-        <v>-58.454849</v>
-      </c>
-      <c r="N174" t="n">
-        <v>-34.559562</v>
-      </c>
-      <c r="O174" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P174" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q174" t="inlineStr">
-        <is>
-          <t>BLO-O</t>
-        </is>
-      </c>
-      <c r="R174" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>-814</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>OLAZABAL AV. 4545</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>814125673</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K175" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L175" t="n">
-        <v>1</v>
-      </c>
-      <c r="M175" t="n">
-        <v>-58.480067</v>
-      </c>
-      <c r="N175" t="n">
-        <v>-34.573072</v>
-      </c>
-      <c r="O175" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P175" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q175" t="inlineStr">
-        <is>
-          <t>ATH-E</t>
-        </is>
-      </c>
-      <c r="R175" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>-816</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>PINTO 4609</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>814125678</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L176" t="n">
-        <v>1</v>
-      </c>
-      <c r="M176" t="n">
-        <v>-58.481182</v>
-      </c>
-      <c r="N176" t="n">
-        <v>-34.544737</v>
-      </c>
-      <c r="O176" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P176" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q176" t="inlineStr">
-        <is>
-          <t>COG-Q</t>
-        </is>
-      </c>
-      <c r="R176" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>